<commit_message>
Rapport du 21 Février 2026
</commit_message>
<xml_diff>
--- a/Donnees_RZ.xlsx
+++ b/Donnees_RZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NDAO ABDOULAYE\Desktop\AFRIKA LEYRI\Rapport\Promoteur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EEF774C-9014-4324-A414-4BD8DCA2BF61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDEECCF3-21AD-44CE-9743-4C80BA997F58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" tabRatio="470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="132">
   <si>
     <t>Date</t>
   </si>
@@ -424,6 +424,12 @@
   </si>
   <si>
     <t>Il réclame le pot de 200g</t>
+  </si>
+  <si>
+    <t>Ibrahima DIALLO (GAMBIEN)</t>
+  </si>
+  <si>
+    <t>Il dit qu'il va exporter le café Altimo stick a gambiee</t>
   </si>
 </sst>
 </file>
@@ -491,7 +497,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -511,6 +517,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -829,8 +844,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}" name="Semaine_1" displayName="Semaine_1" ref="A1:P70" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16">
-  <autoFilter ref="A1:P70" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}" name="Semaine_1" displayName="Semaine_1" ref="A1:P71" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16">
+  <autoFilter ref="A1:P71" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{F85C405C-E78B-4DA6-8568-08107D7551E4}" name="Date" dataDxfId="15"/>
     <tableColumn id="2" xr3:uid="{24A95AD6-D6B8-4864-9451-50BFB3565C62}" name="Prenom_Nom_RZ" dataDxfId="14"/>
@@ -1143,7 +1158,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Feuil2"/>
-  <dimension ref="A1:P70"/>
+  <dimension ref="A1:P71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.53125" bestFit="1" customWidth="1"/>
@@ -1256,11 +1271,11 @@
       <c r="N2" s="10">
         <v>201000</v>
       </c>
-      <c r="O2" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P2" s="12" t="str">
+      <c r="O2" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P2" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1308,11 +1323,11 @@
       <c r="N3" s="10">
         <v>2250000</v>
       </c>
-      <c r="O3" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P3" s="12" t="str">
+      <c r="O3" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P3" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1360,11 +1375,11 @@
       <c r="N4" s="10">
         <v>225000</v>
       </c>
-      <c r="O4" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P4" s="12" t="str">
+      <c r="O4" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P4" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1412,11 +1427,11 @@
       <c r="N5" s="10">
         <v>104000</v>
       </c>
-      <c r="O5" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P5" s="12" t="str">
+      <c r="O5" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P5" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1464,11 +1479,11 @@
       <c r="N6" s="10">
         <v>30000</v>
       </c>
-      <c r="O6" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P6" s="12" t="str">
+      <c r="O6" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P6" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1516,11 +1531,11 @@
       <c r="N7" s="10">
         <v>268000</v>
       </c>
-      <c r="O7" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P7" s="12" t="str">
+      <c r="O7" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P7" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1568,11 +1583,11 @@
       <c r="N8" s="10">
         <v>270000</v>
       </c>
-      <c r="O8" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P8" s="12" t="str">
+      <c r="O8" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P8" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1620,11 +1635,11 @@
       <c r="N9" s="10">
         <v>250000</v>
       </c>
-      <c r="O9" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P9" s="12" t="str">
+      <c r="O9" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P9" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1672,11 +1687,11 @@
       <c r="N10" s="10">
         <v>277500</v>
       </c>
-      <c r="O10" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P10" s="12" t="str">
+      <c r="O10" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P10" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1724,11 +1739,11 @@
       <c r="N11" s="10">
         <v>90000</v>
       </c>
-      <c r="O11" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P11" s="12" t="str">
+      <c r="O11" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P11" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1776,11 +1791,11 @@
       <c r="N12" s="10">
         <v>134000</v>
       </c>
-      <c r="O12" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P12" s="12" t="str">
+      <c r="O12" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P12" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1828,11 +1843,11 @@
       <c r="N13" s="10">
         <v>201000</v>
       </c>
-      <c r="O13" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P13" s="12" t="str">
+      <c r="O13" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P13" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1880,11 +1895,11 @@
       <c r="N14" s="10">
         <v>92500</v>
       </c>
-      <c r="O14" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P14" s="12" t="str">
+      <c r="O14" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P14" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1932,11 +1947,11 @@
       <c r="N15" s="10">
         <v>46250</v>
       </c>
-      <c r="O15" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P15" s="12" t="str">
+      <c r="O15" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P15" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -1984,11 +1999,11 @@
       <c r="N16" s="10">
         <v>270000</v>
       </c>
-      <c r="O16" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P16" s="12" t="str">
+      <c r="O16" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P16" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2036,11 +2051,11 @@
       <c r="N17" s="10">
         <v>450000</v>
       </c>
-      <c r="O17" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P17" s="12" t="str">
+      <c r="O17" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P17" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2088,11 +2103,11 @@
       <c r="N18" s="10">
         <v>450000</v>
       </c>
-      <c r="O18" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P18" s="12" t="str">
+      <c r="O18" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P18" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2140,11 +2155,11 @@
       <c r="N19" s="10">
         <v>936000</v>
       </c>
-      <c r="O19" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P19" s="12" t="str">
+      <c r="O19" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P19" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2192,11 +2207,11 @@
       <c r="N20" s="10">
         <v>450000</v>
       </c>
-      <c r="O20" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P20" s="12" t="str">
+      <c r="O20" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P20" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2244,11 +2259,11 @@
       <c r="N21" s="10">
         <v>33500</v>
       </c>
-      <c r="O21" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P21" s="12" t="str">
+      <c r="O21" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P21" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2296,11 +2311,11 @@
       <c r="N22" s="10">
         <v>250000</v>
       </c>
-      <c r="O22" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P22" s="12" t="str">
+      <c r="O22" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P22" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2348,11 +2363,11 @@
       <c r="N23" s="10">
         <v>67000</v>
       </c>
-      <c r="O23" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P23" s="12" t="str">
+      <c r="O23" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P23" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2400,11 +2415,11 @@
       <c r="N24" s="10">
         <v>268750</v>
       </c>
-      <c r="O24" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P24" s="12" t="str">
+      <c r="O24" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P24" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2452,11 +2467,11 @@
       <c r="N25" s="10">
         <v>150000</v>
       </c>
-      <c r="O25" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P25" s="12" t="str">
+      <c r="O25" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P25" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2504,11 +2519,11 @@
       <c r="N26" s="10">
         <v>33500</v>
       </c>
-      <c r="O26" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P26" s="12" t="str">
+      <c r="O26" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P26" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2556,11 +2571,11 @@
       <c r="N27" s="10">
         <v>537500</v>
       </c>
-      <c r="O27" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P27" s="12" t="str">
+      <c r="O27" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P27" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2608,11 +2623,11 @@
       <c r="N28" s="10">
         <v>180000</v>
       </c>
-      <c r="O28" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P28" s="12" t="str">
+      <c r="O28" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P28" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2660,11 +2675,11 @@
       <c r="N29" s="10">
         <v>9250</v>
       </c>
-      <c r="O29" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P29" s="12" t="str">
+      <c r="O29" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P29" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2712,11 +2727,11 @@
       <c r="N30" s="10">
         <v>9250</v>
       </c>
-      <c r="O30" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P30" s="12" t="str">
+      <c r="O30" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P30" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2764,11 +2779,11 @@
       <c r="N31" s="10">
         <v>9250</v>
       </c>
-      <c r="O31" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P31" s="12" t="str">
+      <c r="O31" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P31" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2816,11 +2831,11 @@
       <c r="N32" s="10">
         <v>9250</v>
       </c>
-      <c r="O32" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P32" s="12" t="str">
+      <c r="O32" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P32" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2868,11 +2883,11 @@
       <c r="N33" s="10">
         <v>12000</v>
       </c>
-      <c r="O33" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P33" s="12" t="str">
+      <c r="O33" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P33" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2920,11 +2935,11 @@
       <c r="N34" s="10">
         <v>650000</v>
       </c>
-      <c r="O34" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P34" s="12" t="str">
+      <c r="O34" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P34" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -2972,11 +2987,11 @@
       <c r="N35" s="10">
         <v>650000</v>
       </c>
-      <c r="O35" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P35" s="12" t="str">
+      <c r="O35" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P35" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3024,11 +3039,11 @@
       <c r="N36" s="10">
         <v>2600000</v>
       </c>
-      <c r="O36" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P36" s="12" t="str">
+      <c r="O36" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P36" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3076,11 +3091,11 @@
       <c r="N37" s="10">
         <v>1000000</v>
       </c>
-      <c r="O37" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P37" s="12" t="str">
+      <c r="O37" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P37" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3128,11 +3143,11 @@
       <c r="N38" s="10">
         <v>22000</v>
       </c>
-      <c r="O38" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P38" s="12" t="str">
+      <c r="O38" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P38" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3180,11 +3195,11 @@
       <c r="N39" s="10">
         <v>36000</v>
       </c>
-      <c r="O39" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P39" s="12" t="str">
+      <c r="O39" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P39" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3232,11 +3247,11 @@
       <c r="N40" s="10">
         <v>36000</v>
       </c>
-      <c r="O40" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P40" s="12" t="str">
+      <c r="O40" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P40" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3284,11 +3299,11 @@
       <c r="N41" s="10">
         <v>250000</v>
       </c>
-      <c r="O41" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P41" s="12" t="str">
+      <c r="O41" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P41" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3336,11 +3351,11 @@
       <c r="N42" s="10">
         <v>520000</v>
       </c>
-      <c r="O42" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P42" s="12" t="str">
+      <c r="O42" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P42" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3388,11 +3403,11 @@
       <c r="N43" s="10">
         <v>150000</v>
       </c>
-      <c r="O43" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P43" s="12" t="str">
+      <c r="O43" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P43" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3440,11 +3455,11 @@
       <c r="N44" s="10">
         <v>60000</v>
       </c>
-      <c r="O44" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P44" s="12" t="str">
+      <c r="O44" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P44" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3492,11 +3507,11 @@
       <c r="N45" s="10">
         <v>54000</v>
       </c>
-      <c r="O45" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P45" s="12" t="str">
+      <c r="O45" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P45" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3544,11 +3559,11 @@
       <c r="N46" s="10">
         <v>2600000</v>
       </c>
-      <c r="O46" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P46" s="12" t="str">
+      <c r="O46" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P46" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3596,11 +3611,11 @@
       <c r="N47" s="10">
         <v>650000</v>
       </c>
-      <c r="O47" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P47" s="12" t="str">
+      <c r="O47" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P47" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3648,11 +3663,11 @@
       <c r="N48" s="10">
         <v>500000</v>
       </c>
-      <c r="O48" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P48" s="12" t="str">
+      <c r="O48" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P48" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3700,11 +3715,11 @@
       <c r="N49" s="10">
         <v>210000</v>
       </c>
-      <c r="O49" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P49" s="12" t="str">
+      <c r="O49" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P49" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3752,11 +3767,11 @@
       <c r="N50" s="10">
         <v>52000</v>
       </c>
-      <c r="O50" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P50" s="12" t="str">
+      <c r="O50" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P50" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3804,11 +3819,11 @@
       <c r="N51" s="10">
         <v>2600000</v>
       </c>
-      <c r="O51" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P51" s="12" t="str">
+      <c r="O51" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P51" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3856,11 +3871,11 @@
       <c r="N52" s="10">
         <v>150000</v>
       </c>
-      <c r="O52" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P52" s="12" t="str">
+      <c r="O52" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P52" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3908,11 +3923,11 @@
       <c r="N53" s="10">
         <v>243750</v>
       </c>
-      <c r="O53" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P53" s="12" t="str">
+      <c r="O53" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P53" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -3960,11 +3975,11 @@
       <c r="N54" s="10">
         <v>231250</v>
       </c>
-      <c r="O54" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P54" s="12" t="str">
+      <c r="O54" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P54" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4012,11 +4027,11 @@
       <c r="N55" s="10">
         <v>600000</v>
       </c>
-      <c r="O55" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P55" s="12" t="str">
+      <c r="O55" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P55" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4064,11 +4079,11 @@
       <c r="N56" s="10">
         <v>243750</v>
       </c>
-      <c r="O56" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P56" s="12" t="str">
+      <c r="O56" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P56" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4116,11 +4131,11 @@
       <c r="N57" s="10">
         <v>19500</v>
       </c>
-      <c r="O57" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P57" s="12" t="str">
+      <c r="O57" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P57" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4168,11 +4183,11 @@
       <c r="N58" s="10">
         <v>234500</v>
       </c>
-      <c r="O58" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P58" s="12" t="str">
+      <c r="O58" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P58" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4220,11 +4235,11 @@
       <c r="N59" s="10">
         <v>240000</v>
       </c>
-      <c r="O59" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P59" s="12" t="str">
+      <c r="O59" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P59" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4272,11 +4287,11 @@
       <c r="N60" s="10">
         <v>243750</v>
       </c>
-      <c r="O60" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P60" s="12" t="str">
+      <c r="O60" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P60" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4324,11 +4339,11 @@
       <c r="N61" s="10">
         <v>97500</v>
       </c>
-      <c r="O61" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P61" s="12" t="str">
+      <c r="O61" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P61" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4376,11 +4391,11 @@
       <c r="N62" s="10">
         <v>33500</v>
       </c>
-      <c r="O62" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P62" s="12" t="str">
+      <c r="O62" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P62" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4428,11 +4443,11 @@
       <c r="N63" s="10">
         <v>33500</v>
       </c>
-      <c r="O63" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P63" s="12" t="str">
+      <c r="O63" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P63" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4480,11 +4495,11 @@
       <c r="N64" s="10">
         <v>24000</v>
       </c>
-      <c r="O64" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P64" s="12" t="str">
+      <c r="O64" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P64" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4532,11 +4547,11 @@
       <c r="N65" s="10">
         <v>30000</v>
       </c>
-      <c r="O65" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P65" s="12" t="str">
+      <c r="O65" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P65" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4584,11 +4599,11 @@
       <c r="N66" s="10">
         <v>36000</v>
       </c>
-      <c r="O66" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P66" s="12" t="str">
+      <c r="O66" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P66" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4636,11 +4651,11 @@
       <c r="N67" s="10">
         <v>750000</v>
       </c>
-      <c r="O67" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P67" s="12" t="str">
+      <c r="O67" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P67" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4688,11 +4703,11 @@
       <c r="N68" s="10">
         <v>450000</v>
       </c>
-      <c r="O68" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P68" s="12" t="str">
+      <c r="O68" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P68" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4740,11 +4755,11 @@
       <c r="N69" s="10">
         <v>650000</v>
       </c>
-      <c r="O69" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P69" s="12" t="str">
+      <c r="O69" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P69" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
@@ -4792,11 +4807,63 @@
       <c r="N70" s="10">
         <v>750000</v>
       </c>
-      <c r="O70" s="11" t="str">
-        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
-        <v>S08</v>
-      </c>
-      <c r="P70" s="12" t="str">
+      <c r="O70" s="7" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P70" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>février</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A71" s="11">
+        <v>46069</v>
+      </c>
+      <c r="B71" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C71" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D71" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E71" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F71" s="12">
+        <v>777032455</v>
+      </c>
+      <c r="G71" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H71" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I71" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J71" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="K71" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="L71" s="12">
+        <v>100</v>
+      </c>
+      <c r="M71" s="13">
+        <v>29500</v>
+      </c>
+      <c r="N71" s="13">
+        <v>2950000</v>
+      </c>
+      <c r="O71" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S08</v>
+      </c>
+      <c r="P71" s="15" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>

</xml_diff>

<commit_message>
Rapport du 07  Mars 2026
</commit_message>
<xml_diff>
--- a/Donnees_RZ.xlsx
+++ b/Donnees_RZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NDAO ABDOULAYE\Desktop\AFRIKA LEYRI\Rapport\Promoteur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0DDFA74-6429-4533-AA9C-38120FC067E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41E5B0F0-AB3B-4131-A0C0-092A21B3668F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" tabRatio="470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1042" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="185">
   <si>
     <t>Date</t>
   </si>
@@ -550,6 +550,45 @@
   </si>
   <si>
     <t>AITA SARR</t>
+  </si>
+  <si>
+    <t>Boubacar BA</t>
+  </si>
+  <si>
+    <t>MOUSTAPHA DIALLO</t>
+  </si>
+  <si>
+    <t>ABLAYE DIALLO</t>
+  </si>
+  <si>
+    <t>Dalifort</t>
+  </si>
+  <si>
+    <t>Sow</t>
+  </si>
+  <si>
+    <t>Grand Dakar</t>
+  </si>
+  <si>
+    <t>Wane</t>
+  </si>
+  <si>
+    <t>HLM</t>
+  </si>
+  <si>
+    <t>Baye sy</t>
+  </si>
+  <si>
+    <t>Moustapha Mbaye</t>
+  </si>
+  <si>
+    <t>Bassirou NDAO</t>
+  </si>
+  <si>
+    <t>Demain stp</t>
+  </si>
+  <si>
+    <t>Moussa</t>
   </si>
 </sst>
 </file>
@@ -905,16 +944,16 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
+        <top style="thin">
           <color auto="1"/>
-        </bottom>
+        </top>
       </border>
     </dxf>
     <dxf>
       <border outline="0">
-        <top style="thin">
+        <bottom style="thin">
           <color auto="1"/>
-        </top>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -964,8 +1003,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}" name="Semaine_1" displayName="Semaine_1" ref="A1:P115" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="16" tableBorderDxfId="17">
-  <autoFilter ref="A1:P115" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}" name="Semaine_1" displayName="Semaine_1" ref="A1:P136" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16">
+  <autoFilter ref="A1:P136" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{F85C405C-E78B-4DA6-8568-08107D7551E4}" name="Date" dataDxfId="15"/>
     <tableColumn id="2" xr3:uid="{24A95AD6-D6B8-4864-9451-50BFB3565C62}" name="Prenom_Nom_RZ" dataDxfId="14"/>
@@ -1278,7 +1317,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Feuil2"/>
-  <dimension ref="A1:P115"/>
+  <dimension ref="A1:P136"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.53125" bestFit="1" customWidth="1"/>
@@ -4989,2291 +5028,3383 @@
       </c>
     </row>
     <row r="72" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A72" s="11">
+      <c r="A72" s="8">
         <v>46076</v>
       </c>
-      <c r="B72" s="12" t="s">
+      <c r="B72" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C72" s="12" t="s">
+      <c r="C72" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D72" s="12" t="s">
+      <c r="D72" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E72" s="12" t="s">
+      <c r="E72" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="F72" s="12">
+      <c r="F72" s="9">
         <v>776428218</v>
       </c>
-      <c r="G72" s="12" t="s">
+      <c r="G72" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H72" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I72" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J72" s="12" t="s">
+      <c r="H72" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I72" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J72" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K72" s="12" t="s">
+      <c r="K72" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L72" s="12">
+      <c r="L72" s="9">
         <v>20</v>
       </c>
-      <c r="M72" s="13">
+      <c r="M72" s="10">
         <v>9500</v>
       </c>
-      <c r="N72" s="13">
+      <c r="N72" s="10">
         <v>190000</v>
       </c>
-      <c r="O72" s="14" t="str">
+      <c r="O72" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P72" s="15" t="str">
+      <c r="P72" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="73" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A73" s="11">
+      <c r="A73" s="8">
         <v>46076</v>
       </c>
-      <c r="B73" s="12" t="s">
+      <c r="B73" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C73" s="12" t="s">
+      <c r="C73" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D73" s="12" t="s">
+      <c r="D73" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E73" s="12" t="s">
+      <c r="E73" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="F73" s="12">
+      <c r="F73" s="9">
         <v>774277399</v>
       </c>
-      <c r="G73" s="12" t="s">
+      <c r="G73" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H73" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I73" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J73" s="12" t="s">
+      <c r="H73" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I73" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J73" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K73" s="12" t="s">
+      <c r="K73" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L73" s="12">
+      <c r="L73" s="9">
         <v>20</v>
       </c>
-      <c r="M73" s="13">
+      <c r="M73" s="10">
         <v>9500</v>
       </c>
-      <c r="N73" s="13">
+      <c r="N73" s="10">
         <v>190000</v>
       </c>
-      <c r="O73" s="14" t="str">
+      <c r="O73" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P73" s="15" t="str">
+      <c r="P73" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="74" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A74" s="11">
+      <c r="A74" s="8">
         <v>46076</v>
       </c>
-      <c r="B74" s="12" t="s">
+      <c r="B74" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C74" s="12" t="s">
+      <c r="C74" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D74" s="12" t="s">
+      <c r="D74" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="E74" s="12" t="s">
+      <c r="E74" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="F74" s="12">
+      <c r="F74" s="9">
         <v>778579191</v>
       </c>
-      <c r="G74" s="12" t="s">
+      <c r="G74" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H74" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I74" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J74" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="K74" s="12" t="s">
+      <c r="H74" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I74" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J74" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K74" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L74" s="12">
+      <c r="L74" s="9">
         <v>30</v>
       </c>
-      <c r="M74" s="13">
+      <c r="M74" s="10">
         <v>9750</v>
       </c>
-      <c r="N74" s="13">
+      <c r="N74" s="10">
         <v>292500</v>
       </c>
-      <c r="O74" s="14" t="str">
+      <c r="O74" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P74" s="15" t="str">
+      <c r="P74" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="75" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A75" s="11">
+      <c r="A75" s="8">
         <v>46076</v>
       </c>
-      <c r="B75" s="12" t="s">
+      <c r="B75" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C75" s="12" t="s">
+      <c r="C75" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D75" s="12" t="s">
+      <c r="D75" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="E75" s="12" t="s">
+      <c r="E75" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="F75" s="12">
+      <c r="F75" s="9">
         <v>774414059</v>
       </c>
-      <c r="G75" s="12" t="s">
+      <c r="G75" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H75" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I75" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J75" s="12" t="s">
+      <c r="H75" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I75" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J75" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="K75" s="12" t="s">
+      <c r="K75" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="L75" s="12">
+      <c r="L75" s="9">
         <v>25</v>
       </c>
-      <c r="M75" s="13">
+      <c r="M75" s="10">
         <v>9250</v>
       </c>
-      <c r="N75" s="13">
+      <c r="N75" s="10">
         <v>231250</v>
       </c>
-      <c r="O75" s="14" t="str">
+      <c r="O75" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P75" s="15" t="str">
+      <c r="P75" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="76" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A76" s="11">
+      <c r="A76" s="8">
         <v>46076</v>
       </c>
-      <c r="B76" s="12" t="s">
+      <c r="B76" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C76" s="12" t="s">
+      <c r="C76" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D76" s="12" t="s">
+      <c r="D76" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="E76" s="12" t="s">
+      <c r="E76" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="F76" s="12">
+      <c r="F76" s="9">
         <v>779486095</v>
       </c>
-      <c r="G76" s="12" t="s">
+      <c r="G76" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H76" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I76" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J76" s="12" t="s">
+      <c r="H76" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I76" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J76" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="K76" s="12" t="s">
+      <c r="K76" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="L76" s="12">
+      <c r="L76" s="9">
         <v>25</v>
       </c>
-      <c r="M76" s="13">
+      <c r="M76" s="10">
         <v>18000</v>
       </c>
-      <c r="N76" s="13">
+      <c r="N76" s="10">
         <v>450000</v>
       </c>
-      <c r="O76" s="14" t="str">
+      <c r="O76" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P76" s="15" t="str">
+      <c r="P76" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="77" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A77" s="11">
+      <c r="A77" s="8">
         <v>46076</v>
       </c>
-      <c r="B77" s="12" t="s">
+      <c r="B77" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C77" s="12" t="s">
+      <c r="C77" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D77" s="12" t="s">
+      <c r="D77" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="E77" s="12" t="s">
+      <c r="E77" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="F77" s="12">
+      <c r="F77" s="9">
         <v>779676016</v>
       </c>
-      <c r="G77" s="12" t="s">
+      <c r="G77" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H77" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I77" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J77" s="12" t="s">
+      <c r="H77" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I77" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J77" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="K77" s="12" t="s">
+      <c r="K77" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L77" s="12">
+      <c r="L77" s="9">
         <v>50</v>
       </c>
-      <c r="M77" s="13">
+      <c r="M77" s="10">
         <v>11000</v>
       </c>
-      <c r="N77" s="13">
+      <c r="N77" s="10">
         <v>550000</v>
       </c>
-      <c r="O77" s="14" t="str">
+      <c r="O77" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P77" s="15" t="str">
+      <c r="P77" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="78" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A78" s="11">
+      <c r="A78" s="8">
         <v>46076</v>
       </c>
-      <c r="B78" s="12" t="s">
+      <c r="B78" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C78" s="12" t="s">
+      <c r="C78" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D78" s="12" t="s">
+      <c r="D78" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E78" s="12" t="s">
+      <c r="E78" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="F78" s="12">
+      <c r="F78" s="9">
         <v>786323232</v>
       </c>
-      <c r="G78" s="12" t="s">
+      <c r="G78" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H78" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I78" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J78" s="12" t="s">
+      <c r="H78" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I78" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J78" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K78" s="12" t="s">
+      <c r="K78" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="L78" s="12">
+      <c r="L78" s="9">
         <v>25</v>
       </c>
-      <c r="M78" s="13">
+      <c r="M78" s="10">
         <v>9250</v>
       </c>
-      <c r="N78" s="13">
+      <c r="N78" s="10">
         <v>231250</v>
       </c>
-      <c r="O78" s="14" t="str">
+      <c r="O78" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P78" s="15" t="str">
+      <c r="P78" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="79" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A79" s="11">
+      <c r="A79" s="8">
         <v>46076</v>
       </c>
-      <c r="B79" s="12" t="s">
+      <c r="B79" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C79" s="12" t="s">
+      <c r="C79" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D79" s="12" t="s">
+      <c r="D79" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="E79" s="12" t="s">
+      <c r="E79" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="F79" s="12">
+      <c r="F79" s="9">
         <v>768059355</v>
       </c>
-      <c r="G79" s="12" t="s">
+      <c r="G79" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H79" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I79" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J79" s="12" t="s">
+      <c r="H79" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I79" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J79" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K79" s="12" t="s">
+      <c r="K79" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L79" s="12">
+      <c r="L79" s="9">
         <v>60</v>
       </c>
-      <c r="M79" s="13">
+      <c r="M79" s="10">
         <v>9500</v>
       </c>
-      <c r="N79" s="13">
+      <c r="N79" s="10">
         <v>570000</v>
       </c>
-      <c r="O79" s="14" t="str">
+      <c r="O79" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P79" s="15" t="str">
+      <c r="P79" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A80" s="11">
+      <c r="A80" s="8">
         <v>46076</v>
       </c>
-      <c r="B80" s="12" t="s">
+      <c r="B80" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C80" s="12" t="s">
+      <c r="C80" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D80" s="12" t="s">
+      <c r="D80" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E80" s="12" t="s">
+      <c r="E80" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="F80" s="12">
+      <c r="F80" s="9">
         <v>773817561</v>
       </c>
-      <c r="G80" s="12" t="s">
+      <c r="G80" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H80" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I80" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J80" s="12" t="s">
+      <c r="H80" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I80" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J80" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="K80" s="12" t="s">
+      <c r="K80" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="L80" s="12">
+      <c r="L80" s="9">
         <v>1</v>
       </c>
-      <c r="M80" s="13">
+      <c r="M80" s="10">
         <v>33500</v>
       </c>
-      <c r="N80" s="13">
+      <c r="N80" s="10">
         <v>33500</v>
       </c>
-      <c r="O80" s="14" t="str">
+      <c r="O80" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P80" s="15" t="str">
+      <c r="P80" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="81" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A81" s="11">
+      <c r="A81" s="8">
         <v>46076</v>
       </c>
-      <c r="B81" s="12" t="s">
+      <c r="B81" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C81" s="12" t="s">
+      <c r="C81" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D81" s="12" t="s">
+      <c r="D81" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E81" s="12" t="s">
+      <c r="E81" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="F81" s="12">
+      <c r="F81" s="9">
         <v>773817561</v>
       </c>
-      <c r="G81" s="12" t="s">
+      <c r="G81" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H81" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I81" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J81" s="12" t="s">
+      <c r="H81" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I81" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J81" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="K81" s="12" t="s">
+      <c r="K81" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L81" s="12">
+      <c r="L81" s="9">
         <v>7</v>
       </c>
-      <c r="M81" s="13">
+      <c r="M81" s="10">
         <v>12000</v>
       </c>
-      <c r="N81" s="13">
+      <c r="N81" s="10">
         <v>84000</v>
       </c>
-      <c r="O81" s="14" t="str">
+      <c r="O81" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P81" s="15" t="str">
+      <c r="P81" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="82" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A82" s="11">
+      <c r="A82" s="8">
         <v>46076</v>
       </c>
-      <c r="B82" s="12" t="s">
+      <c r="B82" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C82" s="12" t="s">
+      <c r="C82" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D82" s="12" t="s">
+      <c r="D82" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E82" s="12" t="s">
+      <c r="E82" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="F82" s="12">
+      <c r="F82" s="9">
         <v>777096402</v>
       </c>
-      <c r="G82" s="12" t="s">
+      <c r="G82" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H82" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I82" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J82" s="12" t="s">
+      <c r="H82" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I82" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J82" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K82" s="12" t="s">
+      <c r="K82" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L82" s="12">
+      <c r="L82" s="9">
         <v>10</v>
       </c>
-      <c r="M82" s="13">
+      <c r="M82" s="10">
         <v>9750</v>
       </c>
-      <c r="N82" s="13">
+      <c r="N82" s="10">
         <v>97500</v>
       </c>
-      <c r="O82" s="14" t="str">
+      <c r="O82" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P82" s="15" t="str">
+      <c r="P82" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A83" s="11">
+      <c r="A83" s="8">
         <v>46076</v>
       </c>
-      <c r="B83" s="12" t="s">
+      <c r="B83" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C83" s="12" t="s">
+      <c r="C83" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D83" s="12" t="s">
+      <c r="D83" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E83" s="12" t="s">
+      <c r="E83" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="F83" s="12">
+      <c r="F83" s="9">
         <v>777096402</v>
       </c>
-      <c r="G83" s="12" t="s">
+      <c r="G83" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H83" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I83" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J83" s="12" t="s">
+      <c r="H83" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I83" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J83" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K83" s="12" t="s">
+      <c r="K83" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L83" s="12">
+      <c r="L83" s="9">
         <v>10</v>
       </c>
-      <c r="M83" s="13">
+      <c r="M83" s="10">
         <v>9750</v>
       </c>
-      <c r="N83" s="13">
+      <c r="N83" s="10">
         <v>97500</v>
       </c>
-      <c r="O83" s="14" t="str">
+      <c r="O83" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P83" s="15" t="str">
+      <c r="P83" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="84" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A84" s="11">
+      <c r="A84" s="8">
         <v>46076</v>
       </c>
-      <c r="B84" s="12" t="s">
+      <c r="B84" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C84" s="12" t="s">
+      <c r="C84" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D84" s="12" t="s">
+      <c r="D84" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E84" s="12" t="s">
+      <c r="E84" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="F84" s="12">
+      <c r="F84" s="9">
         <v>777262311</v>
       </c>
-      <c r="G84" s="12" t="s">
+      <c r="G84" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H84" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I84" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J84" s="12" t="s">
+      <c r="H84" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I84" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J84" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K84" s="12" t="s">
+      <c r="K84" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L84" s="12">
+      <c r="L84" s="9">
         <v>5</v>
       </c>
-      <c r="M84" s="13">
+      <c r="M84" s="10">
         <v>9750</v>
       </c>
-      <c r="N84" s="13">
+      <c r="N84" s="10">
         <v>48750</v>
       </c>
-      <c r="O84" s="14" t="str">
+      <c r="O84" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P84" s="15" t="str">
+      <c r="P84" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="85" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A85" s="11">
+      <c r="A85" s="8">
         <v>46076</v>
       </c>
-      <c r="B85" s="12" t="s">
+      <c r="B85" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C85" s="12" t="s">
+      <c r="C85" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D85" s="12" t="s">
+      <c r="D85" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E85" s="12" t="s">
+      <c r="E85" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="F85" s="12">
+      <c r="F85" s="9">
         <v>777262311</v>
       </c>
-      <c r="G85" s="12" t="s">
+      <c r="G85" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H85" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I85" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J85" s="12" t="s">
+      <c r="H85" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I85" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J85" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K85" s="12" t="s">
+      <c r="K85" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L85" s="12">
+      <c r="L85" s="9">
         <v>5</v>
       </c>
-      <c r="M85" s="13">
+      <c r="M85" s="10">
         <v>12000</v>
       </c>
-      <c r="N85" s="13">
+      <c r="N85" s="10">
         <v>60000</v>
       </c>
-      <c r="O85" s="14" t="str">
+      <c r="O85" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P85" s="15" t="str">
+      <c r="P85" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="86" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A86" s="11">
+      <c r="A86" s="8">
         <v>46078</v>
       </c>
-      <c r="B86" s="12" t="s">
+      <c r="B86" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="C86" s="12" t="s">
+      <c r="C86" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D86" s="12" t="s">
+      <c r="D86" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="E86" s="12" t="s">
+      <c r="E86" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="F86" s="12">
+      <c r="F86" s="9">
         <v>775039973</v>
       </c>
-      <c r="G86" s="12" t="s">
+      <c r="G86" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H86" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I86" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J86" s="12" t="s">
+      <c r="H86" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I86" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J86" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="K86" s="12" t="s">
+      <c r="K86" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L86" s="12">
+      <c r="L86" s="9">
         <v>25</v>
       </c>
-      <c r="M86" s="13">
+      <c r="M86" s="10">
         <v>26000</v>
       </c>
-      <c r="N86" s="13">
+      <c r="N86" s="10">
         <v>650000</v>
       </c>
-      <c r="O86" s="14" t="str">
+      <c r="O86" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P86" s="15" t="str">
+      <c r="P86" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="87" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A87" s="11">
+      <c r="A87" s="8">
         <v>46078</v>
       </c>
-      <c r="B87" s="12" t="s">
+      <c r="B87" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="C87" s="12" t="s">
+      <c r="C87" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D87" s="12" t="s">
+      <c r="D87" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E87" s="12" t="s">
+      <c r="E87" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="F87" s="12">
+      <c r="F87" s="9">
         <v>778356666</v>
       </c>
-      <c r="G87" s="12" t="s">
+      <c r="G87" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H87" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I87" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J87" s="12" t="s">
+      <c r="H87" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I87" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J87" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K87" s="12" t="s">
+      <c r="K87" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L87" s="12">
+      <c r="L87" s="9">
         <v>25</v>
       </c>
-      <c r="M87" s="13">
+      <c r="M87" s="10">
         <v>26000</v>
       </c>
-      <c r="N87" s="13">
+      <c r="N87" s="10">
         <v>650000</v>
       </c>
-      <c r="O87" s="14" t="str">
+      <c r="O87" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P87" s="15" t="str">
+      <c r="P87" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="88" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A88" s="11">
+      <c r="A88" s="8">
         <v>46078</v>
       </c>
-      <c r="B88" s="12" t="s">
+      <c r="B88" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C88" s="12" t="s">
+      <c r="C88" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D88" s="12" t="s">
+      <c r="D88" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E88" s="12" t="s">
+      <c r="E88" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="F88" s="12">
+      <c r="F88" s="9">
         <v>777972938</v>
       </c>
-      <c r="G88" s="12" t="s">
+      <c r="G88" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H88" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I88" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J88" s="12" t="s">
+      <c r="H88" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I88" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J88" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="K88" s="12" t="s">
+      <c r="K88" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L88" s="12">
+      <c r="L88" s="9">
         <v>3</v>
       </c>
-      <c r="M88" s="13">
+      <c r="M88" s="10">
         <v>12000</v>
       </c>
-      <c r="N88" s="13">
+      <c r="N88" s="10">
         <v>36000</v>
       </c>
-      <c r="O88" s="14" t="str">
+      <c r="O88" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P88" s="15" t="str">
+      <c r="P88" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="89" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A89" s="11">
+      <c r="A89" s="8">
         <v>46078</v>
       </c>
-      <c r="B89" s="12" t="s">
+      <c r="B89" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C89" s="12" t="s">
+      <c r="C89" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D89" s="12" t="s">
+      <c r="D89" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E89" s="12" t="s">
+      <c r="E89" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="F89" s="12">
+      <c r="F89" s="9">
         <v>777972938</v>
       </c>
-      <c r="G89" s="12" t="s">
+      <c r="G89" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H89" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I89" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J89" s="12" t="s">
+      <c r="H89" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I89" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J89" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="K89" s="12" t="s">
+      <c r="K89" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="L89" s="12">
+      <c r="L89" s="9">
         <v>2</v>
       </c>
-      <c r="M89" s="13">
+      <c r="M89" s="10">
         <v>33500</v>
       </c>
-      <c r="N89" s="13">
+      <c r="N89" s="10">
         <v>67000</v>
       </c>
-      <c r="O89" s="14" t="str">
+      <c r="O89" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P89" s="15" t="str">
+      <c r="P89" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="90" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A90" s="11">
+      <c r="A90" s="8">
         <v>46078</v>
       </c>
-      <c r="B90" s="12" t="s">
+      <c r="B90" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C90" s="12" t="s">
+      <c r="C90" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D90" s="12" t="s">
+      <c r="D90" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E90" s="12" t="s">
+      <c r="E90" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="F90" s="12">
+      <c r="F90" s="9">
         <v>777972938</v>
       </c>
-      <c r="G90" s="12" t="s">
+      <c r="G90" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H90" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I90" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J90" s="12" t="s">
+      <c r="H90" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I90" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J90" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="K90" s="12" t="s">
+      <c r="K90" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="L90" s="12">
+      <c r="L90" s="9">
         <v>2</v>
       </c>
-      <c r="M90" s="13">
+      <c r="M90" s="10">
         <v>33500</v>
       </c>
-      <c r="N90" s="13">
+      <c r="N90" s="10">
         <v>67000</v>
       </c>
-      <c r="O90" s="14" t="str">
+      <c r="O90" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P90" s="15" t="str">
+      <c r="P90" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="91" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A91" s="11">
+      <c r="A91" s="8">
         <v>46078</v>
       </c>
-      <c r="B91" s="12" t="s">
+      <c r="B91" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C91" s="12" t="s">
+      <c r="C91" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D91" s="12" t="s">
+      <c r="D91" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E91" s="12" t="s">
+      <c r="E91" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="F91" s="12">
+      <c r="F91" s="9">
         <v>777972938</v>
       </c>
-      <c r="G91" s="12" t="s">
+      <c r="G91" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H91" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I91" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J91" s="12" t="s">
+      <c r="H91" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I91" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J91" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="K91" s="12" t="s">
+      <c r="K91" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="L91" s="12">
+      <c r="L91" s="9">
         <v>1</v>
       </c>
-      <c r="M91" s="13">
+      <c r="M91" s="10">
         <v>17500</v>
       </c>
-      <c r="N91" s="13">
+      <c r="N91" s="10">
         <v>17500</v>
       </c>
-      <c r="O91" s="14" t="str">
+      <c r="O91" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P91" s="15" t="str">
+      <c r="P91" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="92" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A92" s="11">
+      <c r="A92" s="8">
         <v>46078</v>
       </c>
-      <c r="B92" s="12" t="s">
+      <c r="B92" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C92" s="12" t="s">
+      <c r="C92" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D92" s="12" t="s">
+      <c r="D92" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E92" s="12" t="s">
+      <c r="E92" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="F92" s="12">
+      <c r="F92" s="9">
         <v>777972938</v>
       </c>
-      <c r="G92" s="12" t="s">
+      <c r="G92" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H92" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I92" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J92" s="12" t="s">
+      <c r="H92" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I92" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J92" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="K92" s="12" t="s">
+      <c r="K92" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L92" s="12">
+      <c r="L92" s="9">
         <v>2</v>
       </c>
-      <c r="M92" s="13">
+      <c r="M92" s="10">
         <v>26000</v>
       </c>
-      <c r="N92" s="13">
+      <c r="N92" s="10">
         <v>52000</v>
       </c>
-      <c r="O92" s="14" t="str">
+      <c r="O92" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P92" s="15" t="str">
+      <c r="P92" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="93" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A93" s="11">
+      <c r="A93" s="8">
         <v>46078</v>
       </c>
-      <c r="B93" s="12" t="s">
+      <c r="B93" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C93" s="12" t="s">
+      <c r="C93" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D93" s="12" t="s">
+      <c r="D93" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E93" s="12" t="s">
+      <c r="E93" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F93" s="12">
+      <c r="F93" s="9">
         <v>775894235</v>
       </c>
-      <c r="G93" s="12" t="s">
+      <c r="G93" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H93" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I93" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J93" s="12" t="s">
+      <c r="H93" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I93" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J93" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="K93" s="12" t="s">
+      <c r="K93" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L93" s="12">
+      <c r="L93" s="9">
         <v>25</v>
       </c>
-      <c r="M93" s="13">
+      <c r="M93" s="10">
         <v>12000</v>
       </c>
-      <c r="N93" s="13">
+      <c r="N93" s="10">
         <v>300000</v>
       </c>
-      <c r="O93" s="14" t="str">
+      <c r="O93" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P93" s="15" t="str">
+      <c r="P93" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="94" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A94" s="11">
+      <c r="A94" s="8">
         <v>46078</v>
       </c>
-      <c r="B94" s="12" t="s">
+      <c r="B94" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="C94" s="12" t="s">
+      <c r="C94" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D94" s="12" t="s">
+      <c r="D94" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="E94" s="12" t="s">
+      <c r="E94" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="F94" s="12">
+      <c r="F94" s="9">
         <v>774379845</v>
       </c>
-      <c r="G94" s="12" t="s">
+      <c r="G94" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H94" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I94" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J94" s="12" t="s">
+      <c r="H94" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I94" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J94" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="K94" s="12" t="s">
+      <c r="K94" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L94" s="12">
+      <c r="L94" s="9">
         <v>25</v>
       </c>
-      <c r="M94" s="13">
+      <c r="M94" s="10">
         <v>26000</v>
       </c>
-      <c r="N94" s="13">
+      <c r="N94" s="10">
         <v>650000</v>
       </c>
-      <c r="O94" s="14" t="str">
+      <c r="O94" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P94" s="15" t="str">
+      <c r="P94" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="95" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A95" s="11">
+      <c r="A95" s="8">
         <v>46078</v>
       </c>
-      <c r="B95" s="12" t="s">
+      <c r="B95" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="C95" s="12" t="s">
+      <c r="C95" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D95" s="12" t="s">
+      <c r="D95" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E95" s="12" t="s">
+      <c r="E95" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="F95" s="12">
+      <c r="F95" s="9">
         <v>778356666</v>
       </c>
-      <c r="G95" s="12" t="s">
+      <c r="G95" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H95" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I95" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J95" s="12" t="s">
+      <c r="H95" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I95" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J95" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K95" s="12" t="s">
+      <c r="K95" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="L95" s="12">
+      <c r="L95" s="9">
         <v>5</v>
       </c>
-      <c r="M95" s="13">
+      <c r="M95" s="10">
         <v>18000</v>
       </c>
-      <c r="N95" s="13">
+      <c r="N95" s="10">
         <v>90000</v>
       </c>
-      <c r="O95" s="14" t="str">
+      <c r="O95" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P95" s="15" t="str">
+      <c r="P95" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="96" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A96" s="11">
+      <c r="A96" s="8">
         <v>46078</v>
       </c>
-      <c r="B96" s="12" t="s">
+      <c r="B96" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="C96" s="12" t="s">
+      <c r="C96" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D96" s="12" t="s">
+      <c r="D96" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E96" s="12" t="s">
+      <c r="E96" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="F96" s="12">
+      <c r="F96" s="9">
         <v>778356666</v>
       </c>
-      <c r="G96" s="12" t="s">
+      <c r="G96" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H96" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I96" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J96" s="12" t="s">
+      <c r="H96" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I96" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J96" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K96" s="12" t="s">
+      <c r="K96" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="L96" s="12">
+      <c r="L96" s="9">
         <v>2</v>
       </c>
-      <c r="M96" s="13">
+      <c r="M96" s="10">
         <v>18000</v>
       </c>
-      <c r="N96" s="13">
+      <c r="N96" s="10">
         <v>36000</v>
       </c>
-      <c r="O96" s="14" t="str">
+      <c r="O96" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P96" s="15" t="str">
+      <c r="P96" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="97" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A97" s="11">
+      <c r="A97" s="8">
         <v>46079</v>
       </c>
-      <c r="B97" s="12" t="s">
+      <c r="B97" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C97" s="12" t="s">
+      <c r="C97" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D97" s="12" t="s">
+      <c r="D97" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="E97" s="12" t="s">
+      <c r="E97" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="F97" s="12">
+      <c r="F97" s="9">
         <v>774061052</v>
       </c>
-      <c r="G97" s="12" t="s">
+      <c r="G97" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H97" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I97" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J97" s="12" t="s">
+      <c r="H97" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I97" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J97" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K97" s="12" t="s">
+      <c r="K97" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L97" s="12">
+      <c r="L97" s="9">
         <v>50</v>
       </c>
-      <c r="M97" s="13">
+      <c r="M97" s="10">
         <v>26000</v>
       </c>
-      <c r="N97" s="13">
+      <c r="N97" s="10">
         <v>1300000</v>
       </c>
-      <c r="O97" s="14" t="str">
+      <c r="O97" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P97" s="15" t="str">
+      <c r="P97" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="98" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A98" s="11">
+      <c r="A98" s="8">
         <v>46079</v>
       </c>
-      <c r="B98" s="12" t="s">
+      <c r="B98" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C98" s="12" t="s">
+      <c r="C98" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D98" s="12" t="s">
+      <c r="D98" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="E98" s="12" t="s">
+      <c r="E98" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="F98" s="12">
+      <c r="F98" s="9">
         <v>774446240</v>
       </c>
-      <c r="G98" s="12" t="s">
+      <c r="G98" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H98" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I98" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J98" s="12" t="s">
+      <c r="H98" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I98" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J98" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="K98" s="12" t="s">
+      <c r="K98" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="L98" s="12">
+      <c r="L98" s="9">
         <v>25</v>
       </c>
-      <c r="M98" s="13">
+      <c r="M98" s="10">
         <v>9250</v>
       </c>
-      <c r="N98" s="13">
+      <c r="N98" s="10">
         <v>231250</v>
       </c>
-      <c r="O98" s="14" t="str">
+      <c r="O98" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P98" s="15" t="str">
+      <c r="P98" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="99" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A99" s="11">
+      <c r="A99" s="8">
         <v>46079</v>
       </c>
-      <c r="B99" s="12" t="s">
+      <c r="B99" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C99" s="12" t="s">
+      <c r="C99" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D99" s="12" t="s">
+      <c r="D99" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E99" s="12" t="s">
+      <c r="E99" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F99" s="12">
+      <c r="F99" s="9">
         <v>774245132</v>
       </c>
-      <c r="G99" s="12" t="s">
+      <c r="G99" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H99" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I99" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J99" s="12" t="s">
+      <c r="H99" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I99" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J99" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K99" s="12" t="s">
+      <c r="K99" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L99" s="12">
+      <c r="L99" s="9">
         <v>25</v>
       </c>
-      <c r="M99" s="13">
+      <c r="M99" s="10">
         <v>26000</v>
       </c>
-      <c r="N99" s="13">
+      <c r="N99" s="10">
         <v>650000</v>
       </c>
-      <c r="O99" s="14" t="str">
+      <c r="O99" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P99" s="15" t="str">
+      <c r="P99" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="100" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A100" s="11">
+      <c r="A100" s="8">
         <v>46079</v>
       </c>
-      <c r="B100" s="12" t="s">
+      <c r="B100" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C100" s="12" t="s">
+      <c r="C100" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D100" s="12" t="s">
+      <c r="D100" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="E100" s="12" t="s">
+      <c r="E100" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="F100" s="12">
+      <c r="F100" s="9">
         <v>773777037</v>
       </c>
-      <c r="G100" s="12" t="s">
+      <c r="G100" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H100" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I100" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J100" s="12" t="s">
+      <c r="H100" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I100" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J100" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K100" s="12" t="s">
+      <c r="K100" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L100" s="12">
+      <c r="L100" s="9">
         <v>25</v>
       </c>
-      <c r="M100" s="13">
+      <c r="M100" s="10">
         <v>26000</v>
       </c>
-      <c r="N100" s="13">
+      <c r="N100" s="10">
         <v>650000</v>
       </c>
-      <c r="O100" s="14" t="str">
+      <c r="O100" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P100" s="15" t="str">
+      <c r="P100" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="101" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A101" s="11">
+      <c r="A101" s="8">
         <v>46079</v>
       </c>
-      <c r="B101" s="12" t="s">
+      <c r="B101" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="C101" s="12" t="s">
+      <c r="C101" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D101" s="12" t="s">
+      <c r="D101" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="E101" s="12" t="s">
+      <c r="E101" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="F101" s="12">
+      <c r="F101" s="9">
         <v>774216339</v>
       </c>
-      <c r="G101" s="12" t="s">
+      <c r="G101" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H101" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I101" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J101" s="12" t="s">
+      <c r="H101" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I101" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J101" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K101" s="12" t="s">
+      <c r="K101" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L101" s="12">
+      <c r="L101" s="9">
         <v>25</v>
       </c>
-      <c r="M101" s="13">
+      <c r="M101" s="10">
         <v>26000</v>
       </c>
-      <c r="N101" s="13">
+      <c r="N101" s="10">
         <v>650000</v>
       </c>
-      <c r="O101" s="14" t="str">
+      <c r="O101" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P101" s="15" t="str">
+      <c r="P101" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="102" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A102" s="11">
+      <c r="A102" s="8">
         <v>46079</v>
       </c>
-      <c r="B102" s="12" t="s">
+      <c r="B102" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C102" s="12" t="s">
+      <c r="C102" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D102" s="12" t="s">
+      <c r="D102" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E102" s="12" t="s">
+      <c r="E102" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="F102" s="12">
+      <c r="F102" s="9">
         <v>772289185</v>
       </c>
-      <c r="G102" s="12" t="s">
+      <c r="G102" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H102" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I102" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J102" s="12" t="s">
+      <c r="H102" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I102" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J102" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K102" s="12" t="s">
+      <c r="K102" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L102" s="12">
+      <c r="L102" s="9">
         <v>25</v>
       </c>
-      <c r="M102" s="13">
+      <c r="M102" s="10">
         <v>26000</v>
       </c>
-      <c r="N102" s="13">
+      <c r="N102" s="10">
         <v>650000</v>
       </c>
-      <c r="O102" s="14" t="str">
+      <c r="O102" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P102" s="15" t="str">
+      <c r="P102" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="103" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A103" s="11">
+      <c r="A103" s="8">
         <v>46079</v>
       </c>
-      <c r="B103" s="12" t="s">
+      <c r="B103" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C103" s="12" t="s">
+      <c r="C103" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D103" s="12" t="s">
+      <c r="D103" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E103" s="12" t="s">
+      <c r="E103" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="F103" s="12">
+      <c r="F103" s="9">
         <v>772289185</v>
       </c>
-      <c r="G103" s="12" t="s">
+      <c r="G103" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H103" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I103" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J103" s="12" t="s">
+      <c r="H103" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I103" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J103" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K103" s="12" t="s">
+      <c r="K103" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="L103" s="12">
+      <c r="L103" s="9">
         <v>1</v>
       </c>
-      <c r="M103" s="13">
+      <c r="M103" s="10">
         <v>17500</v>
       </c>
-      <c r="N103" s="13">
+      <c r="N103" s="10">
         <v>17500</v>
       </c>
-      <c r="O103" s="14" t="str">
+      <c r="O103" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P103" s="15" t="str">
+      <c r="P103" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="104" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A104" s="11">
+      <c r="A104" s="8">
         <v>46079</v>
       </c>
-      <c r="B104" s="12" t="s">
+      <c r="B104" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C104" s="12" t="s">
+      <c r="C104" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D104" s="12" t="s">
+      <c r="D104" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E104" s="12" t="s">
+      <c r="E104" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="F104" s="12">
+      <c r="F104" s="9">
         <v>772289185</v>
       </c>
-      <c r="G104" s="12" t="s">
+      <c r="G104" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H104" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I104" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J104" s="12" t="s">
+      <c r="H104" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I104" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J104" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K104" s="12" t="s">
+      <c r="K104" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="L104" s="12">
+      <c r="L104" s="9">
         <v>3</v>
       </c>
-      <c r="M104" s="13">
+      <c r="M104" s="10">
         <v>9250</v>
       </c>
-      <c r="N104" s="13">
+      <c r="N104" s="10">
         <v>27750</v>
       </c>
-      <c r="O104" s="14" t="str">
+      <c r="O104" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P104" s="15" t="str">
+      <c r="P104" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="105" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A105" s="11">
+      <c r="A105" s="8">
         <v>46079</v>
       </c>
-      <c r="B105" s="12" t="s">
+      <c r="B105" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C105" s="12" t="s">
+      <c r="C105" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D105" s="12" t="s">
+      <c r="D105" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E105" s="12" t="s">
+      <c r="E105" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="F105" s="12">
+      <c r="F105" s="9">
         <v>772289185</v>
       </c>
-      <c r="G105" s="12" t="s">
+      <c r="G105" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H105" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I105" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J105" s="12" t="s">
+      <c r="H105" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I105" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J105" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K105" s="12" t="s">
+      <c r="K105" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="L105" s="12">
+      <c r="L105" s="9">
         <v>1</v>
       </c>
-      <c r="M105" s="13">
+      <c r="M105" s="10">
         <v>18000</v>
       </c>
-      <c r="N105" s="13">
+      <c r="N105" s="10">
         <v>18000</v>
       </c>
-      <c r="O105" s="14" t="str">
+      <c r="O105" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P105" s="15" t="str">
+      <c r="P105" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="106" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A106" s="11">
+      <c r="A106" s="8">
         <v>46079</v>
       </c>
-      <c r="B106" s="12" t="s">
+      <c r="B106" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C106" s="12" t="s">
+      <c r="C106" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D106" s="12" t="s">
+      <c r="D106" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="E106" s="12" t="s">
+      <c r="E106" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="F106" s="12">
+      <c r="F106" s="9">
         <v>771355863</v>
       </c>
-      <c r="G106" s="12" t="s">
+      <c r="G106" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H106" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I106" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J106" s="12" t="s">
+      <c r="H106" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I106" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J106" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="K106" s="12" t="s">
+      <c r="K106" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L106" s="12">
+      <c r="L106" s="9">
         <v>25</v>
       </c>
-      <c r="M106" s="13">
+      <c r="M106" s="10">
         <v>26000</v>
       </c>
-      <c r="N106" s="13">
+      <c r="N106" s="10">
         <v>650000</v>
       </c>
-      <c r="O106" s="14" t="str">
+      <c r="O106" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P106" s="15" t="str">
+      <c r="P106" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="107" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A107" s="11">
+      <c r="A107" s="8">
         <v>46079</v>
       </c>
-      <c r="B107" s="12" t="s">
+      <c r="B107" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="C107" s="12" t="s">
+      <c r="C107" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D107" s="12" t="s">
+      <c r="D107" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="E107" s="12" t="s">
+      <c r="E107" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="F107" s="12">
+      <c r="F107" s="9">
         <v>783596501</v>
       </c>
-      <c r="G107" s="12" t="s">
+      <c r="G107" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="H107" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I107" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J107" s="12" t="s">
+      <c r="H107" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I107" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J107" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="K107" s="12" t="s">
+      <c r="K107" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L107" s="12">
+      <c r="L107" s="9">
         <v>1</v>
       </c>
-      <c r="M107" s="13">
+      <c r="M107" s="10">
         <v>26000</v>
       </c>
-      <c r="N107" s="13">
+      <c r="N107" s="10">
         <v>26000</v>
       </c>
-      <c r="O107" s="14" t="str">
+      <c r="O107" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P107" s="15" t="str">
+      <c r="P107" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="108" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A108" s="11">
+      <c r="A108" s="8">
         <v>46079</v>
       </c>
-      <c r="B108" s="12" t="s">
+      <c r="B108" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="C108" s="12" t="s">
+      <c r="C108" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D108" s="12" t="s">
+      <c r="D108" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="E108" s="12" t="s">
+      <c r="E108" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="F108" s="12">
+      <c r="F108" s="9">
         <v>783596501</v>
       </c>
-      <c r="G108" s="12" t="s">
+      <c r="G108" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="H108" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I108" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J108" s="12" t="s">
+      <c r="H108" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I108" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J108" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="K108" s="12" t="s">
+      <c r="K108" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="L108" s="12">
+      <c r="L108" s="9">
         <v>2</v>
       </c>
-      <c r="M108" s="13">
+      <c r="M108" s="10">
         <v>9250</v>
       </c>
-      <c r="N108" s="13">
+      <c r="N108" s="10">
         <v>18500</v>
       </c>
-      <c r="O108" s="14" t="str">
+      <c r="O108" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P108" s="15" t="str">
+      <c r="P108" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="109" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A109" s="11">
+      <c r="A109" s="8">
         <v>46079</v>
       </c>
-      <c r="B109" s="12" t="s">
+      <c r="B109" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="C109" s="12" t="s">
+      <c r="C109" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D109" s="12" t="s">
+      <c r="D109" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="E109" s="12" t="s">
+      <c r="E109" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="F109" s="12">
+      <c r="F109" s="9">
         <v>761760410</v>
       </c>
-      <c r="G109" s="12" t="s">
+      <c r="G109" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="H109" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I109" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J109" s="12" t="s">
+      <c r="H109" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I109" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J109" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="K109" s="12" t="s">
+      <c r="K109" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="L109" s="12">
+      <c r="L109" s="9">
         <v>1</v>
       </c>
-      <c r="M109" s="13">
+      <c r="M109" s="10">
         <v>9250</v>
       </c>
-      <c r="N109" s="13">
+      <c r="N109" s="10">
         <v>9250</v>
       </c>
-      <c r="O109" s="14" t="str">
+      <c r="O109" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P109" s="15" t="str">
+      <c r="P109" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="110" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A110" s="11">
+      <c r="A110" s="8">
         <v>46079</v>
       </c>
-      <c r="B110" s="12" t="s">
+      <c r="B110" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="C110" s="12" t="s">
+      <c r="C110" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="D110" s="12" t="s">
+      <c r="D110" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="E110" s="12" t="s">
+      <c r="E110" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="F110" s="12">
+      <c r="F110" s="9">
         <v>761760410</v>
       </c>
-      <c r="G110" s="12" t="s">
+      <c r="G110" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="H110" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I110" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J110" s="12" t="s">
+      <c r="H110" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I110" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J110" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="K110" s="12" t="s">
+      <c r="K110" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L110" s="12">
+      <c r="L110" s="9">
         <v>1</v>
       </c>
-      <c r="M110" s="13">
+      <c r="M110" s="10">
         <v>12000</v>
       </c>
-      <c r="N110" s="13">
+      <c r="N110" s="10">
         <v>12000</v>
       </c>
-      <c r="O110" s="14" t="str">
+      <c r="O110" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P110" s="15" t="str">
+      <c r="P110" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="111" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A111" s="11">
+      <c r="A111" s="8">
         <v>46080</v>
       </c>
-      <c r="B111" s="12" t="s">
+      <c r="B111" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C111" s="12" t="s">
+      <c r="C111" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D111" s="12" t="s">
+      <c r="D111" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E111" s="12" t="s">
+      <c r="E111" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="F111" s="12">
+      <c r="F111" s="9">
         <v>776175166</v>
       </c>
-      <c r="G111" s="12" t="s">
+      <c r="G111" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H111" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I111" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J111" s="12" t="s">
+      <c r="H111" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I111" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J111" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="K111" s="12" t="s">
+      <c r="K111" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L111" s="12">
+      <c r="L111" s="9">
         <v>100</v>
       </c>
-      <c r="M111" s="13">
+      <c r="M111" s="10">
         <v>26000</v>
       </c>
-      <c r="N111" s="13">
+      <c r="N111" s="10">
         <v>2600000</v>
       </c>
-      <c r="O111" s="14" t="str">
+      <c r="O111" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P111" s="15" t="str">
+      <c r="P111" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="112" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A112" s="11">
+      <c r="A112" s="8">
         <v>46079</v>
       </c>
-      <c r="B112" s="12" t="s">
+      <c r="B112" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C112" s="12" t="s">
+      <c r="C112" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D112" s="12" t="s">
+      <c r="D112" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E112" s="12" t="s">
+      <c r="E112" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="F112" s="12">
+      <c r="F112" s="9">
         <v>773817561</v>
       </c>
-      <c r="G112" s="12" t="s">
+      <c r="G112" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H112" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I112" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J112" s="12" t="s">
+      <c r="H112" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I112" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J112" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="K112" s="12" t="s">
+      <c r="K112" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="L112" s="12">
+      <c r="L112" s="9">
         <v>31</v>
       </c>
-      <c r="M112" s="13">
+      <c r="M112" s="10">
         <v>6000</v>
       </c>
-      <c r="N112" s="13">
+      <c r="N112" s="10">
         <v>186000</v>
       </c>
-      <c r="O112" s="14" t="str">
+      <c r="O112" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P112" s="15" t="str">
+      <c r="P112" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="113" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A113" s="11">
+      <c r="A113" s="8">
         <v>46079</v>
       </c>
-      <c r="B113" s="12" t="s">
+      <c r="B113" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C113" s="12" t="s">
+      <c r="C113" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D113" s="12" t="s">
+      <c r="D113" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E113" s="12" t="s">
+      <c r="E113" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="F113" s="12">
+      <c r="F113" s="9">
         <v>773817561</v>
       </c>
-      <c r="G113" s="12" t="s">
+      <c r="G113" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H113" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I113" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J113" s="12" t="s">
+      <c r="H113" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I113" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J113" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="K113" s="12" t="s">
+      <c r="K113" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L113" s="12">
+      <c r="L113" s="9">
         <v>3</v>
       </c>
-      <c r="M113" s="13">
+      <c r="M113" s="10">
         <v>26000</v>
       </c>
-      <c r="N113" s="13">
+      <c r="N113" s="10">
         <v>78000</v>
       </c>
-      <c r="O113" s="14" t="str">
+      <c r="O113" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P113" s="15" t="str">
+      <c r="P113" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="114" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A114" s="11">
+      <c r="A114" s="8">
         <v>46079</v>
       </c>
-      <c r="B114" s="12" t="s">
+      <c r="B114" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C114" s="12" t="s">
+      <c r="C114" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D114" s="12" t="s">
+      <c r="D114" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="E114" s="12" t="s">
+      <c r="E114" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="F114" s="12">
+      <c r="F114" s="9">
         <v>775079426</v>
       </c>
-      <c r="G114" s="12" t="s">
+      <c r="G114" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H114" s="12" t="s">
+      <c r="H114" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="I114" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J114" s="12" t="s">
+      <c r="I114" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J114" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="K114" s="12" t="s">
+      <c r="K114" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L114" s="12">
+      <c r="L114" s="9">
         <v>1</v>
       </c>
-      <c r="M114" s="13">
+      <c r="M114" s="10">
         <v>12000</v>
       </c>
-      <c r="N114" s="13">
+      <c r="N114" s="10">
         <v>12000</v>
       </c>
-      <c r="O114" s="14" t="str">
+      <c r="O114" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P114" s="15" t="str">
+      <c r="P114" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>février</v>
       </c>
     </row>
     <row r="115" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A115" s="11">
+      <c r="A115" s="8">
         <v>46079</v>
       </c>
-      <c r="B115" s="12" t="s">
+      <c r="B115" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C115" s="12" t="s">
+      <c r="C115" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D115" s="12" t="s">
+      <c r="D115" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E115" s="12" t="s">
+      <c r="E115" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="F115" s="12">
+      <c r="F115" s="9">
         <v>771166914</v>
       </c>
-      <c r="G115" s="12" t="s">
+      <c r="G115" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H115" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I115" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J115" s="12" t="s">
+      <c r="H115" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I115" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="J115" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="K115" s="12" t="s">
+      <c r="K115" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="L115" s="12">
+      <c r="L115" s="9">
         <v>1</v>
       </c>
-      <c r="M115" s="13">
+      <c r="M115" s="10">
         <v>26000</v>
       </c>
-      <c r="N115" s="13">
+      <c r="N115" s="10">
         <v>26000</v>
       </c>
-      <c r="O115" s="14" t="str">
+      <c r="O115" s="7" t="str">
         <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S09</v>
       </c>
-      <c r="P115" s="15" t="str">
-        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
-        <v>février</v>
+      <c r="P115" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>février</v>
+      </c>
+    </row>
+    <row r="116" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A116" s="11">
+        <v>46083</v>
+      </c>
+      <c r="B116" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C116" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D116" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E116" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="F116" s="12">
+        <v>776712564</v>
+      </c>
+      <c r="G116" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H116" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I116" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J116" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K116" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="L116" s="12">
+        <v>7</v>
+      </c>
+      <c r="M116" s="13">
+        <v>18000</v>
+      </c>
+      <c r="N116" s="13">
+        <v>126000</v>
+      </c>
+      <c r="O116" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P116" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="117" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A117" s="11">
+        <v>46083</v>
+      </c>
+      <c r="B117" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C117" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D117" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E117" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="F117" s="12">
+        <v>776712564</v>
+      </c>
+      <c r="G117" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H117" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I117" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J117" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K117" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="L117" s="12">
+        <v>3</v>
+      </c>
+      <c r="M117" s="13">
+        <v>18000</v>
+      </c>
+      <c r="N117" s="13">
+        <v>54000</v>
+      </c>
+      <c r="O117" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P117" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="118" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A118" s="11">
+        <v>46083</v>
+      </c>
+      <c r="B118" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C118" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D118" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E118" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="F118" s="12">
+        <v>776712564</v>
+      </c>
+      <c r="G118" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H118" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I118" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J118" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K118" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="L118" s="12">
+        <v>1</v>
+      </c>
+      <c r="M118" s="13">
+        <v>9750</v>
+      </c>
+      <c r="N118" s="13">
+        <v>9750</v>
+      </c>
+      <c r="O118" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P118" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="119" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A119" s="11">
+        <v>46083</v>
+      </c>
+      <c r="B119" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C119" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D119" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E119" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="F119" s="12">
+        <v>779676016</v>
+      </c>
+      <c r="G119" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H119" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I119" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J119" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K119" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="L119" s="12">
+        <v>25</v>
+      </c>
+      <c r="M119" s="13">
+        <v>11000</v>
+      </c>
+      <c r="N119" s="13">
+        <v>275000</v>
+      </c>
+      <c r="O119" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P119" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="120" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A120" s="11">
+        <v>46083</v>
+      </c>
+      <c r="B120" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C120" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D120" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="E120" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="F120" s="12">
+        <v>778976507</v>
+      </c>
+      <c r="G120" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H120" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I120" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J120" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="K120" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L120" s="12">
+        <v>25</v>
+      </c>
+      <c r="M120" s="13">
+        <v>26000</v>
+      </c>
+      <c r="N120" s="13">
+        <v>650000</v>
+      </c>
+      <c r="O120" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P120" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="121" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A121" s="11">
+        <v>46083</v>
+      </c>
+      <c r="B121" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C121" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D121" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="E121" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="F121" s="12">
+        <v>771010134</v>
+      </c>
+      <c r="G121" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H121" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I121" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J121" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="K121" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L121" s="12">
+        <v>100</v>
+      </c>
+      <c r="M121" s="13">
+        <v>26000</v>
+      </c>
+      <c r="N121" s="13">
+        <v>2600000</v>
+      </c>
+      <c r="O121" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P121" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="122" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A122" s="11">
+        <v>46084</v>
+      </c>
+      <c r="B122" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C122" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D122" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E122" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="F122" s="12">
+        <v>784537895</v>
+      </c>
+      <c r="G122" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H122" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I122" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J122" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K122" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="L122" s="12">
+        <v>50</v>
+      </c>
+      <c r="M122" s="13">
+        <v>9000</v>
+      </c>
+      <c r="N122" s="13">
+        <v>450000</v>
+      </c>
+      <c r="O122" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P122" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="123" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A123" s="11">
+        <v>46084</v>
+      </c>
+      <c r="B123" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C123" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D123" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E123" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="F123" s="12">
+        <v>775586604</v>
+      </c>
+      <c r="G123" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H123" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I123" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J123" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K123" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="L123" s="12">
+        <v>50</v>
+      </c>
+      <c r="M123" s="13">
+        <v>9000</v>
+      </c>
+      <c r="N123" s="13">
+        <v>450000</v>
+      </c>
+      <c r="O123" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P123" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="124" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A124" s="11">
+        <v>46088</v>
+      </c>
+      <c r="B124" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C124" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D124" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="E124" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="F124" s="12">
+        <v>776172529</v>
+      </c>
+      <c r="G124" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H124" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I124" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J124" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K124" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="L124" s="12">
+        <v>1</v>
+      </c>
+      <c r="M124" s="13">
+        <v>9250</v>
+      </c>
+      <c r="N124" s="13">
+        <v>9250</v>
+      </c>
+      <c r="O124" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P124" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="125" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A125" s="11">
+        <v>46088</v>
+      </c>
+      <c r="B125" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C125" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D125" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="E125" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="F125" s="12">
+        <v>776172529</v>
+      </c>
+      <c r="G125" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H125" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I125" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J125" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K125" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="L125" s="12">
+        <v>1</v>
+      </c>
+      <c r="M125" s="13">
+        <v>17500</v>
+      </c>
+      <c r="N125" s="13">
+        <v>17500</v>
+      </c>
+      <c r="O125" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P125" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="126" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A126" s="11">
+        <v>46088</v>
+      </c>
+      <c r="B126" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C126" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D126" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="E126" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="F126" s="12">
+        <v>776172529</v>
+      </c>
+      <c r="G126" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H126" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I126" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J126" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K126" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="L126" s="12">
+        <v>11</v>
+      </c>
+      <c r="M126" s="13">
+        <v>29000</v>
+      </c>
+      <c r="N126" s="13">
+        <v>319000</v>
+      </c>
+      <c r="O126" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P126" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="127" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A127" s="11">
+        <v>46088</v>
+      </c>
+      <c r="B127" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C127" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D127" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="E127" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="F127" s="12">
+        <v>776172529</v>
+      </c>
+      <c r="G127" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H127" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I127" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J127" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K127" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L127" s="12">
+        <v>14</v>
+      </c>
+      <c r="M127" s="13">
+        <v>26000</v>
+      </c>
+      <c r="N127" s="13">
+        <v>364000</v>
+      </c>
+      <c r="O127" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P127" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="128" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A128" s="11">
+        <v>46087</v>
+      </c>
+      <c r="B128" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C128" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D128" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E128" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="F128" s="12">
+        <v>775273147</v>
+      </c>
+      <c r="G128" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H128" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I128" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J128" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K128" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L128" s="12">
+        <v>1</v>
+      </c>
+      <c r="M128" s="13">
+        <v>26000</v>
+      </c>
+      <c r="N128" s="13">
+        <v>26000</v>
+      </c>
+      <c r="O128" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P128" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="129" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A129" s="11">
+        <v>46087</v>
+      </c>
+      <c r="B129" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C129" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D129" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E129" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="F129" s="12">
+        <v>775273147</v>
+      </c>
+      <c r="G129" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H129" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I129" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J129" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K129" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="L129" s="12">
+        <v>25</v>
+      </c>
+      <c r="M129" s="13">
+        <v>6000</v>
+      </c>
+      <c r="N129" s="13">
+        <v>150000</v>
+      </c>
+      <c r="O129" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P129" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="130" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A130" s="11">
+        <v>46087</v>
+      </c>
+      <c r="B130" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C130" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D130" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="E130" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="F130" s="12">
+        <v>775411988</v>
+      </c>
+      <c r="G130" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H130" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I130" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J130" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K130" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="L130" s="12">
+        <v>4</v>
+      </c>
+      <c r="M130" s="13">
+        <v>33500</v>
+      </c>
+      <c r="N130" s="13">
+        <v>134000</v>
+      </c>
+      <c r="O130" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P130" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="131" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A131" s="11">
+        <v>46087</v>
+      </c>
+      <c r="B131" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C131" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D131" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="E131" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="F131" s="12">
+        <v>775079426</v>
+      </c>
+      <c r="G131" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H131" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I131" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J131" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K131" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="L131" s="12">
+        <v>1</v>
+      </c>
+      <c r="M131" s="13">
+        <v>12000</v>
+      </c>
+      <c r="N131" s="13">
+        <v>12000</v>
+      </c>
+      <c r="O131" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P131" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="132" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A132" s="11">
+        <v>46087</v>
+      </c>
+      <c r="B132" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C132" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D132" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="E132" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="F132" s="12">
+        <v>775014335</v>
+      </c>
+      <c r="G132" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H132" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I132" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J132" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K132" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="L132" s="12">
+        <v>1</v>
+      </c>
+      <c r="M132" s="13">
+        <v>12000</v>
+      </c>
+      <c r="N132" s="13">
+        <v>12000</v>
+      </c>
+      <c r="O132" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P132" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="133" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A133" s="11">
+        <v>46086</v>
+      </c>
+      <c r="B133" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C133" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D133" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E133" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="F133" s="12">
+        <v>772899294</v>
+      </c>
+      <c r="G133" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H133" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I133" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J133" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K133" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L133" s="12">
+        <v>25</v>
+      </c>
+      <c r="M133" s="13">
+        <v>26000</v>
+      </c>
+      <c r="N133" s="13">
+        <v>650000</v>
+      </c>
+      <c r="O133" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P133" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="134" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A134" s="11">
+        <v>46086</v>
+      </c>
+      <c r="B134" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C134" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D134" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E134" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="F134" s="12">
+        <v>775544532</v>
+      </c>
+      <c r="G134" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H134" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I134" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J134" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="K134" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L134" s="12">
+        <v>24</v>
+      </c>
+      <c r="M134" s="13">
+        <v>26000</v>
+      </c>
+      <c r="N134" s="13">
+        <v>624000</v>
+      </c>
+      <c r="O134" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P134" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="135" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A135" s="11">
+        <v>46086</v>
+      </c>
+      <c r="B135" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C135" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D135" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="E135" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="F135" s="12">
+        <v>771837885</v>
+      </c>
+      <c r="G135" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H135" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I135" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J135" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K135" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L135" s="12">
+        <v>1</v>
+      </c>
+      <c r="M135" s="13">
+        <v>26000</v>
+      </c>
+      <c r="N135" s="13">
+        <v>26000</v>
+      </c>
+      <c r="O135" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P135" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
+      </c>
+    </row>
+    <row r="136" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A136" s="11">
+        <v>46086</v>
+      </c>
+      <c r="B136" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C136" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D136" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="E136" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="F136" s="12">
+        <v>771837885</v>
+      </c>
+      <c r="G136" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H136" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I136" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J136" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K136" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="L136" s="12">
+        <v>3</v>
+      </c>
+      <c r="M136" s="13">
+        <v>12000</v>
+      </c>
+      <c r="N136" s="13">
+        <v>36000</v>
+      </c>
+      <c r="O136" s="14" t="str">
+        <f>"S0"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S010</v>
+      </c>
+      <c r="P136" s="15" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mars</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rapport du 18 Avril 2026
</commit_message>
<xml_diff>
--- a/Donnees_RZ.xlsx
+++ b/Donnees_RZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NDAO ABDOULAYE\Desktop\AFRIKA LEYRI\Rapport\Promoteur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{266CE197-01D9-4798-BD59-DC365CBDD749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F39375-4229-4139-892F-2CA51F4F8D1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" tabRatio="470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2482" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2968" uniqueCount="300">
   <si>
     <t>Date</t>
   </si>
@@ -850,6 +850,90 @@
   </si>
   <si>
     <t>Client satisfait</t>
+  </si>
+  <si>
+    <t>Ibrahima</t>
+  </si>
+  <si>
+    <t>Chocolat transparent 200gx24pcs</t>
+  </si>
+  <si>
+    <t>Chocolat transparent 400gx12pcs</t>
+  </si>
+  <si>
+    <t>Meadowlite 25Kg</t>
+  </si>
+  <si>
+    <t>Souhaibou</t>
+  </si>
+  <si>
+    <t>KEUR MASSAR N°2</t>
+  </si>
+  <si>
+    <t>Bayakh</t>
+  </si>
+  <si>
+    <t>Bada THIAW</t>
+  </si>
+  <si>
+    <t>Tournal Yeumbeul</t>
+  </si>
+  <si>
+    <t>ALPHA DIALLO</t>
+  </si>
+  <si>
+    <t>SEYNABOU BA</t>
+  </si>
+  <si>
+    <t>Matar Ndaiye</t>
+  </si>
+  <si>
+    <t>Fallou</t>
+  </si>
+  <si>
+    <t>Chocolat jaune 200g x 24 pcs</t>
+  </si>
+  <si>
+    <t>Khassa Diop</t>
+  </si>
+  <si>
+    <t>Mame  Gor</t>
+  </si>
+  <si>
+    <t>Korka</t>
+  </si>
+  <si>
+    <t>Pa Sylla</t>
+  </si>
+  <si>
+    <t>Idrissa</t>
+  </si>
+  <si>
+    <t>Modou</t>
+  </si>
+  <si>
+    <t>Darro TOURE</t>
+  </si>
+  <si>
+    <t>Tapha</t>
+  </si>
+  <si>
+    <t>Mamodou DIALLO</t>
+  </si>
+  <si>
+    <t>Mactar Diallo</t>
+  </si>
+  <si>
+    <t>Supermarché le cayor</t>
+  </si>
+  <si>
+    <t>Gueye et frère</t>
+  </si>
+  <si>
+    <t>Mamadou DIBA</t>
+  </si>
+  <si>
+    <t>Supermarché</t>
   </si>
 </sst>
 </file>
@@ -917,7 +1001,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -947,6 +1031,22 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1251,8 +1351,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}" name="Semaine_1" displayName="Semaine_1" ref="A1:P275" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16">
-  <autoFilter ref="A1:P275" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}" name="Semaine_1" displayName="Semaine_1" ref="A1:P329" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16">
+  <autoFilter ref="A1:P329" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{F85C405C-E78B-4DA6-8568-08107D7551E4}" name="Date" dataDxfId="15"/>
     <tableColumn id="2" xr3:uid="{24A95AD6-D6B8-4864-9451-50BFB3565C62}" name="Prenom_Nom_RZ" dataDxfId="14"/>
@@ -1565,7 +1665,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Feuil2"/>
-  <dimension ref="A1:P275"/>
+  <dimension ref="A1:P329"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.53125" bestFit="1" customWidth="1"/>
@@ -15883,6 +15983,2814 @@
         <v>avril</v>
       </c>
     </row>
+    <row r="276" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A276" s="11">
+        <v>46125</v>
+      </c>
+      <c r="B276" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="C276" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D276" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="E276" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="F276" s="13">
+        <v>777739323</v>
+      </c>
+      <c r="G276" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H276" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I276" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J276" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K276" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="L276" s="12">
+        <v>30</v>
+      </c>
+      <c r="M276" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N276" s="14">
+        <v>270000</v>
+      </c>
+      <c r="O276" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P276" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="277" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A277" s="11">
+        <v>46125</v>
+      </c>
+      <c r="B277" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="C277" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D277" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="E277" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="F277" s="13">
+        <v>777739323</v>
+      </c>
+      <c r="G277" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H277" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I277" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J277" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K277" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="L277" s="12">
+        <v>3</v>
+      </c>
+      <c r="M277" s="14">
+        <v>28000</v>
+      </c>
+      <c r="N277" s="14">
+        <v>84000</v>
+      </c>
+      <c r="O277" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P277" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="278" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A278" s="11">
+        <v>46125</v>
+      </c>
+      <c r="B278" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="C278" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D278" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E278" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="F278" s="13">
+        <v>779486095</v>
+      </c>
+      <c r="G278" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H278" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I278" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J278" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K278" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="L278" s="12">
+        <v>15</v>
+      </c>
+      <c r="M278" s="14">
+        <v>12500</v>
+      </c>
+      <c r="N278" s="14">
+        <v>187500</v>
+      </c>
+      <c r="O278" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P278" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="279" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A279" s="11">
+        <v>46125</v>
+      </c>
+      <c r="B279" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="C279" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D279" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E279" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="F279" s="13">
+        <v>779486095</v>
+      </c>
+      <c r="G279" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H279" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I279" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J279" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K279" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="L279" s="12">
+        <v>10</v>
+      </c>
+      <c r="M279" s="14">
+        <v>12500</v>
+      </c>
+      <c r="N279" s="14">
+        <v>125000</v>
+      </c>
+      <c r="O279" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P279" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="280" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A280" s="11">
+        <v>46125</v>
+      </c>
+      <c r="B280" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C280" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D280" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E280" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="F280" s="13">
+        <v>778356666</v>
+      </c>
+      <c r="G280" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H280" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I280" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J280" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K280" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L280" s="12">
+        <v>25</v>
+      </c>
+      <c r="M280" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N280" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O280" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P280" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="281" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A281" s="11">
+        <v>46125</v>
+      </c>
+      <c r="B281" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C281" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D281" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="E281" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="F281" s="13">
+        <v>774216339</v>
+      </c>
+      <c r="G281" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H281" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I281" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J281" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="K281" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L281" s="12">
+        <v>50</v>
+      </c>
+      <c r="M281" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N281" s="14">
+        <v>1300000</v>
+      </c>
+      <c r="O281" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P281" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="282" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A282" s="11">
+        <v>46125</v>
+      </c>
+      <c r="B282" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C282" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D282" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="E282" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="F282" s="13">
+        <v>774216339</v>
+      </c>
+      <c r="G282" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H282" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I282" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J282" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="K282" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="L282" s="12">
+        <v>5</v>
+      </c>
+      <c r="M282" s="14">
+        <v>19500</v>
+      </c>
+      <c r="N282" s="14">
+        <v>97500</v>
+      </c>
+      <c r="O282" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P282" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="283" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A283" s="11">
+        <v>46125</v>
+      </c>
+      <c r="B283" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C283" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D283" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E283" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="F283" s="13">
+        <v>776634479</v>
+      </c>
+      <c r="G283" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H283" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I283" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J283" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="K283" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="L283" s="12">
+        <v>25</v>
+      </c>
+      <c r="M283" s="14">
+        <v>53000</v>
+      </c>
+      <c r="N283" s="14">
+        <v>1325000</v>
+      </c>
+      <c r="O283" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P283" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="284" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A284" s="11">
+        <v>46125</v>
+      </c>
+      <c r="B284" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C284" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D284" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E284" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="F284" s="13">
+        <v>774624747</v>
+      </c>
+      <c r="G284" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H284" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I284" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J284" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="K284" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="L284" s="12">
+        <v>20</v>
+      </c>
+      <c r="M284" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N284" s="14">
+        <v>180000</v>
+      </c>
+      <c r="O284" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P284" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="285" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A285" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B285" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C285" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D285" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="E285" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="F285" s="13">
+        <v>779598695</v>
+      </c>
+      <c r="G285" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H285" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I285" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J285" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="K285" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L285" s="12">
+        <v>25</v>
+      </c>
+      <c r="M285" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N285" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O285" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P285" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="286" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A286" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B286" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C286" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D286" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="E286" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="F286" s="13">
+        <v>773531341</v>
+      </c>
+      <c r="G286" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H286" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I286" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J286" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K286" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="L286" s="12">
+        <v>1</v>
+      </c>
+      <c r="M286" s="14">
+        <v>53000</v>
+      </c>
+      <c r="N286" s="14">
+        <v>53000</v>
+      </c>
+      <c r="O286" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P286" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="287" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A287" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B287" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C287" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D287" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="E287" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="F287" s="13">
+        <v>775586819</v>
+      </c>
+      <c r="G287" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H287" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I287" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J287" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K287" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L287" s="12">
+        <v>25</v>
+      </c>
+      <c r="M287" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N287" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O287" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P287" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="288" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A288" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B288" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C288" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D288" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="E288" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="F288" s="13">
+        <v>768059355</v>
+      </c>
+      <c r="G288" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H288" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I288" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J288" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K288" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="L288" s="12">
+        <v>50</v>
+      </c>
+      <c r="M288" s="14">
+        <v>28000</v>
+      </c>
+      <c r="N288" s="14">
+        <v>1400000</v>
+      </c>
+      <c r="O288" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P288" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="289" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A289" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B289" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="C289" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="D289" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="E289" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="F289" s="13">
+        <v>763639555</v>
+      </c>
+      <c r="G289" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H289" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I289" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J289" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K289" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="L289" s="12">
+        <v>1</v>
+      </c>
+      <c r="M289" s="14">
+        <v>17500</v>
+      </c>
+      <c r="N289" s="14">
+        <v>17500</v>
+      </c>
+      <c r="O289" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P289" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="290" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A290" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B290" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="C290" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="D290" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="E290" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="F290" s="13">
+        <v>763639555</v>
+      </c>
+      <c r="G290" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H290" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I290" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J290" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K290" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="L290" s="12">
+        <v>26</v>
+      </c>
+      <c r="M290" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N290" s="14">
+        <v>234000</v>
+      </c>
+      <c r="O290" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P290" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="291" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A291" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B291" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="C291" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="D291" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="E291" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="F291" s="13">
+        <v>763639555</v>
+      </c>
+      <c r="G291" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H291" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I291" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J291" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K291" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L291" s="12">
+        <v>9</v>
+      </c>
+      <c r="M291" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N291" s="14">
+        <v>234000</v>
+      </c>
+      <c r="O291" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P291" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="292" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A292" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B292" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C292" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D292" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="E292" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="F292" s="13">
+        <v>778650281</v>
+      </c>
+      <c r="G292" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H292" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I292" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J292" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K292" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L292" s="12">
+        <v>25</v>
+      </c>
+      <c r="M292" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N292" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O292" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P292" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="293" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A293" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B293" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C293" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D293" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="E293" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="F293" s="13">
+        <v>773340367</v>
+      </c>
+      <c r="G293" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H293" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I293" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J293" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K293" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L293" s="12">
+        <v>12</v>
+      </c>
+      <c r="M293" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N293" s="14">
+        <v>312000</v>
+      </c>
+      <c r="O293" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P293" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="294" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A294" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B294" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C294" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D294" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="E294" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="F294" s="13">
+        <v>779420909</v>
+      </c>
+      <c r="G294" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H294" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I294" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J294" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K294" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L294" s="12">
+        <v>13</v>
+      </c>
+      <c r="M294" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N294" s="14">
+        <v>338000</v>
+      </c>
+      <c r="O294" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P294" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="295" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A295" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B295" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C295" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D295" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="E295" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="F295" s="13">
+        <v>768059355</v>
+      </c>
+      <c r="G295" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H295" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I295" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J295" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K295" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="L295" s="12">
+        <v>50</v>
+      </c>
+      <c r="M295" s="14">
+        <v>28000</v>
+      </c>
+      <c r="N295" s="14">
+        <v>1400000</v>
+      </c>
+      <c r="O295" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P295" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="296" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A296" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B296" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C296" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D296" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E296" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="F296" s="13">
+        <v>771165277</v>
+      </c>
+      <c r="G296" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H296" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I296" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J296" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K296" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="L296" s="12">
+        <v>2</v>
+      </c>
+      <c r="M296" s="14">
+        <v>53000</v>
+      </c>
+      <c r="N296" s="14">
+        <v>106000</v>
+      </c>
+      <c r="O296" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P296" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="297" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A297" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B297" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C297" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D297" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E297" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="F297" s="13">
+        <v>763469670</v>
+      </c>
+      <c r="G297" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H297" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I297" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J297" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K297" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="L297" s="12">
+        <v>100</v>
+      </c>
+      <c r="M297" s="14">
+        <v>53000</v>
+      </c>
+      <c r="N297" s="14">
+        <v>5300000</v>
+      </c>
+      <c r="O297" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P297" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="298" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A298" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B298" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C298" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D298" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E298" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="F298" s="13">
+        <v>771786135</v>
+      </c>
+      <c r="G298" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H298" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I298" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J298" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K298" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="L298" s="12">
+        <v>2</v>
+      </c>
+      <c r="M298" s="14">
+        <v>12500</v>
+      </c>
+      <c r="N298" s="14">
+        <v>25000</v>
+      </c>
+      <c r="O298" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P298" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="299" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A299" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B299" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C299" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D299" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E299" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="F299" s="13">
+        <v>771786135</v>
+      </c>
+      <c r="G299" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H299" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I299" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J299" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K299" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="L299" s="12">
+        <v>2</v>
+      </c>
+      <c r="M299" s="14">
+        <v>15500</v>
+      </c>
+      <c r="N299" s="14">
+        <v>31000</v>
+      </c>
+      <c r="O299" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P299" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="300" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A300" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B300" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C300" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D300" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E300" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="F300" s="13">
+        <v>778852859</v>
+      </c>
+      <c r="G300" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H300" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I300" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J300" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K300" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L300" s="12">
+        <v>25</v>
+      </c>
+      <c r="M300" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N300" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O300" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P300" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="301" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A301" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B301" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C301" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D301" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E301" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="F301" s="13">
+        <v>708015391</v>
+      </c>
+      <c r="G301" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H301" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I301" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J301" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K301" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="L301" s="12">
+        <v>1</v>
+      </c>
+      <c r="M301" s="14">
+        <v>53000</v>
+      </c>
+      <c r="N301" s="14">
+        <v>53000</v>
+      </c>
+      <c r="O301" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P301" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="302" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A302" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B302" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C302" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D302" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E302" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="F302" s="13">
+        <v>772131614</v>
+      </c>
+      <c r="G302" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H302" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I302" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J302" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K302" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="L302" s="12">
+        <v>10</v>
+      </c>
+      <c r="M302" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N302" s="14">
+        <v>90000</v>
+      </c>
+      <c r="O302" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P302" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="303" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A303" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B303" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C303" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D303" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E303" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="F303" s="13">
+        <v>778276533</v>
+      </c>
+      <c r="G303" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H303" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I303" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J303" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K303" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L303" s="12">
+        <v>1</v>
+      </c>
+      <c r="M303" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N303" s="14">
+        <v>26000</v>
+      </c>
+      <c r="O303" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P303" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="304" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A304" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B304" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C304" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D304" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E304" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="F304" s="13">
+        <v>775544532</v>
+      </c>
+      <c r="G304" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H304" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I304" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J304" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="K304" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L304" s="12">
+        <v>24</v>
+      </c>
+      <c r="M304" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N304" s="14">
+        <v>624000</v>
+      </c>
+      <c r="O304" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P304" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="305" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A305" s="11">
+        <v>46129</v>
+      </c>
+      <c r="B305" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C305" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D305" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E305" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="F305" s="13">
+        <v>772131614</v>
+      </c>
+      <c r="G305" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H305" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I305" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J305" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K305" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="L305" s="12">
+        <v>1</v>
+      </c>
+      <c r="M305" s="14">
+        <v>53000</v>
+      </c>
+      <c r="N305" s="14">
+        <v>53000</v>
+      </c>
+      <c r="O305" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P305" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="306" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A306" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B306" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C306" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D306" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E306" s="12" t="s">
+        <v>290</v>
+      </c>
+      <c r="F306" s="13">
+        <v>779865100</v>
+      </c>
+      <c r="G306" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H306" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I306" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J306" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="K306" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="L306" s="12">
+        <v>10</v>
+      </c>
+      <c r="M306" s="14">
+        <v>19500</v>
+      </c>
+      <c r="N306" s="14">
+        <v>195000</v>
+      </c>
+      <c r="O306" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P306" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="307" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A307" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B307" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C307" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D307" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E307" s="12" t="s">
+        <v>290</v>
+      </c>
+      <c r="F307" s="13">
+        <v>779865100</v>
+      </c>
+      <c r="G307" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H307" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I307" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J307" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="K307" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="L307" s="12">
+        <v>20</v>
+      </c>
+      <c r="M307" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N307" s="14">
+        <v>180000</v>
+      </c>
+      <c r="O307" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P307" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="308" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A308" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B308" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C308" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D308" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E308" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="F308" s="13">
+        <v>771871533</v>
+      </c>
+      <c r="G308" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H308" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I308" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J308" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K308" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="L308" s="12">
+        <v>1</v>
+      </c>
+      <c r="M308" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N308" s="14">
+        <v>9000</v>
+      </c>
+      <c r="O308" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P308" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="309" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A309" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B309" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C309" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D309" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E309" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="F309" s="13">
+        <v>771871533</v>
+      </c>
+      <c r="G309" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H309" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I309" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J309" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K309" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L309" s="12">
+        <v>5</v>
+      </c>
+      <c r="M309" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N309" s="14">
+        <v>130000</v>
+      </c>
+      <c r="O309" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P309" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="310" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A310" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B310" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C310" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D310" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E310" s="12" t="s">
+        <v>292</v>
+      </c>
+      <c r="F310" s="13">
+        <v>773501029</v>
+      </c>
+      <c r="G310" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H310" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I310" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J310" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K310" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="L310" s="12">
+        <v>1</v>
+      </c>
+      <c r="M310" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N310" s="14">
+        <v>9000</v>
+      </c>
+      <c r="O310" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P310" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="311" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A311" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B311" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C311" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D311" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E311" s="12" t="s">
+        <v>292</v>
+      </c>
+      <c r="F311" s="13">
+        <v>773501029</v>
+      </c>
+      <c r="G311" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H311" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I311" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J311" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K311" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L311" s="12">
+        <v>5</v>
+      </c>
+      <c r="M311" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N311" s="14">
+        <v>130000</v>
+      </c>
+      <c r="O311" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P311" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="312" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A312" s="11">
+        <v>46127</v>
+      </c>
+      <c r="B312" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C312" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D312" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E312" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="F312" s="13">
+        <v>784464768</v>
+      </c>
+      <c r="G312" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H312" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I312" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J312" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="K312" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L312" s="12">
+        <v>16</v>
+      </c>
+      <c r="M312" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N312" s="14">
+        <v>416000</v>
+      </c>
+      <c r="O312" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P312" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="313" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A313" s="11">
+        <v>46126</v>
+      </c>
+      <c r="B313" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C313" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D313" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E313" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="F313" s="13">
+        <v>781316258</v>
+      </c>
+      <c r="G313" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H313" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I313" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J313" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="K313" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L313" s="12">
+        <v>5</v>
+      </c>
+      <c r="M313" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N313" s="14">
+        <v>130000</v>
+      </c>
+      <c r="O313" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P313" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="314" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A314" s="11">
+        <v>46126</v>
+      </c>
+      <c r="B314" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C314" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D314" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E314" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="F314" s="13">
+        <v>775378651</v>
+      </c>
+      <c r="G314" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H314" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I314" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J314" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="K314" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L314" s="12">
+        <v>25</v>
+      </c>
+      <c r="M314" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N314" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O314" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P314" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="315" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A315" s="11">
+        <v>46126</v>
+      </c>
+      <c r="B315" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C315" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D315" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E315" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="F315" s="13">
+        <v>781316258</v>
+      </c>
+      <c r="G315" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H315" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I315" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J315" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="K315" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="L315" s="12">
+        <v>5</v>
+      </c>
+      <c r="M315" s="14">
+        <v>19500</v>
+      </c>
+      <c r="N315" s="14">
+        <v>97500</v>
+      </c>
+      <c r="O315" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P315" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="316" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A316" s="11">
+        <v>46126</v>
+      </c>
+      <c r="B316" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C316" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D316" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E316" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="F316" s="13">
+        <v>781316258</v>
+      </c>
+      <c r="G316" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H316" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I316" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J316" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="K316" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="L316" s="12">
+        <v>10</v>
+      </c>
+      <c r="M316" s="14">
+        <v>28000</v>
+      </c>
+      <c r="N316" s="14">
+        <v>280000</v>
+      </c>
+      <c r="O316" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P316" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="317" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A317" s="11">
+        <v>46126</v>
+      </c>
+      <c r="B317" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C317" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D317" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E317" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="F317" s="13">
+        <v>775378651</v>
+      </c>
+      <c r="G317" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H317" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I317" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J317" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="K317" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="L317" s="12">
+        <v>3</v>
+      </c>
+      <c r="M317" s="14">
+        <v>19500</v>
+      </c>
+      <c r="N317" s="14">
+        <v>58500</v>
+      </c>
+      <c r="O317" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P317" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="318" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A318" s="11">
+        <v>46126</v>
+      </c>
+      <c r="B318" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C318" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D318" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E318" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="F318" s="13">
+        <v>775378651</v>
+      </c>
+      <c r="G318" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H318" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I318" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J318" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="K318" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="L318" s="12">
+        <v>5</v>
+      </c>
+      <c r="M318" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N318" s="14">
+        <v>45000</v>
+      </c>
+      <c r="O318" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P318" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="319" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A319" s="11">
+        <v>46126</v>
+      </c>
+      <c r="B319" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C319" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D319" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E319" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="F319" s="13">
+        <v>775378651</v>
+      </c>
+      <c r="G319" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H319" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I319" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J319" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="K319" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="L319" s="12">
+        <v>10</v>
+      </c>
+      <c r="M319" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N319" s="14">
+        <v>90000</v>
+      </c>
+      <c r="O319" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P319" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="320" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A320" s="11">
+        <v>46126</v>
+      </c>
+      <c r="B320" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C320" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D320" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E320" s="12" t="s">
+        <v>296</v>
+      </c>
+      <c r="F320" s="13">
+        <v>776367168</v>
+      </c>
+      <c r="G320" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H320" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I320" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J320" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K320" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L320" s="12">
+        <v>25</v>
+      </c>
+      <c r="M320" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N320" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O320" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P320" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="321" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A321" s="11">
+        <v>46126</v>
+      </c>
+      <c r="B321" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C321" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D321" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E321" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="F321" s="13">
+        <v>773248259</v>
+      </c>
+      <c r="G321" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="H321" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I321" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J321" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K321" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="L321" s="12">
+        <v>2</v>
+      </c>
+      <c r="M321" s="14">
+        <v>19500</v>
+      </c>
+      <c r="N321" s="14">
+        <v>39000</v>
+      </c>
+      <c r="O321" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P321" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="322" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A322" s="11">
+        <v>46126</v>
+      </c>
+      <c r="B322" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C322" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D322" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E322" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="F322" s="13">
+        <v>774446616</v>
+      </c>
+      <c r="G322" s="12" t="s">
+        <v>299</v>
+      </c>
+      <c r="H322" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I322" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J322" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="K322" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="L322" s="12">
+        <v>4</v>
+      </c>
+      <c r="M322" s="14">
+        <v>12500</v>
+      </c>
+      <c r="N322" s="14">
+        <v>50000</v>
+      </c>
+      <c r="O322" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P322" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="323" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A323" s="11">
+        <v>46126</v>
+      </c>
+      <c r="B323" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C323" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D323" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E323" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="F323" s="13">
+        <v>774446616</v>
+      </c>
+      <c r="G323" s="12" t="s">
+        <v>299</v>
+      </c>
+      <c r="H323" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I323" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J323" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="K323" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="L323" s="12">
+        <v>1</v>
+      </c>
+      <c r="M323" s="14">
+        <v>15500</v>
+      </c>
+      <c r="N323" s="14">
+        <v>15500</v>
+      </c>
+      <c r="O323" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P323" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="324" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A324" s="11">
+        <v>46130</v>
+      </c>
+      <c r="B324" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="C324" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="D324" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="E324" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="F324" s="13">
+        <v>762951288</v>
+      </c>
+      <c r="G324" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H324" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I324" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J324" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K324" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L324" s="12">
+        <v>1</v>
+      </c>
+      <c r="M324" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N324" s="14">
+        <v>26000</v>
+      </c>
+      <c r="O324" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P324" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="325" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A325" s="11">
+        <v>46130</v>
+      </c>
+      <c r="B325" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C325" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D325" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E325" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F325" s="13">
+        <v>772038792</v>
+      </c>
+      <c r="G325" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H325" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I325" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J325" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="K325" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="L325" s="12">
+        <v>1</v>
+      </c>
+      <c r="M325" s="14">
+        <v>53000</v>
+      </c>
+      <c r="N325" s="14">
+        <v>53000</v>
+      </c>
+      <c r="O325" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P325" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="326" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A326" s="11">
+        <v>46130</v>
+      </c>
+      <c r="B326" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C326" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D326" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E326" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F326" s="13">
+        <v>772038792</v>
+      </c>
+      <c r="G326" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H326" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I326" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J326" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="K326" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="L326" s="12">
+        <v>2</v>
+      </c>
+      <c r="M326" s="14">
+        <v>19500</v>
+      </c>
+      <c r="N326" s="14">
+        <v>39000</v>
+      </c>
+      <c r="O326" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P326" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="327" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A327" s="11">
+        <v>46130</v>
+      </c>
+      <c r="B327" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C327" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D327" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E327" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="F327" s="13">
+        <v>774993694</v>
+      </c>
+      <c r="G327" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H327" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I327" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J327" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="K327" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L327" s="12">
+        <v>50</v>
+      </c>
+      <c r="M327" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N327" s="14">
+        <v>1300000</v>
+      </c>
+      <c r="O327" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P327" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="328" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A328" s="11">
+        <v>46130</v>
+      </c>
+      <c r="B328" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="C328" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="D328" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="E328" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="F328" s="13">
+        <v>762951288</v>
+      </c>
+      <c r="G328" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H328" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I328" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J328" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K328" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="L328" s="12">
+        <v>37</v>
+      </c>
+      <c r="M328" s="14">
+        <v>53000</v>
+      </c>
+      <c r="N328" s="14">
+        <v>1961000</v>
+      </c>
+      <c r="O328" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P328" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
+    <row r="329" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A329" s="11">
+        <v>46130</v>
+      </c>
+      <c r="B329" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="C329" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="D329" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="E329" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="F329" s="13">
+        <v>762951288</v>
+      </c>
+      <c r="G329" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H329" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="I329" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J329" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K329" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="L329" s="12">
+        <v>1</v>
+      </c>
+      <c r="M329" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N329" s="14">
+        <v>9000</v>
+      </c>
+      <c r="O329" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S16</v>
+      </c>
+      <c r="P329" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>avril</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rapport du 23 Mai 2026
</commit_message>
<xml_diff>
--- a/Donnees_RZ.xlsx
+++ b/Donnees_RZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NDAO ABDOULAYE\Desktop\AFRIKA LEYRI\Rapport\Promoteur\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16B93793-3C0D-40E7-84CB-547EEF2E2EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522E29B6-FCCD-4E9F-BF98-8C76FFF81394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10996" tabRatio="470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1122" uniqueCount="195">
   <si>
     <t>Date</t>
   </si>
@@ -483,6 +483,141 @@
   </si>
   <si>
     <t xml:space="preserve">Livré hier soir </t>
+  </si>
+  <si>
+    <t>Nd</t>
+  </si>
+  <si>
+    <t>Khadim Lo</t>
+  </si>
+  <si>
+    <t>Il a commencé à vendre le café royal raison pour laquelle il a diminué sa commande</t>
+  </si>
+  <si>
+    <t>Asse</t>
+  </si>
+  <si>
+    <t>Abdourahmane</t>
+  </si>
+  <si>
+    <t>Sakina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Client satisfait </t>
+  </si>
+  <si>
+    <t>Zac Mbao</t>
+  </si>
+  <si>
+    <t>Ibrahima Tahirou</t>
+  </si>
+  <si>
+    <t>Keur Mbaye Fall</t>
+  </si>
+  <si>
+    <t>Pape</t>
+  </si>
+  <si>
+    <t>Abdou</t>
+  </si>
+  <si>
+    <t>Keur Ndiaye LO</t>
+  </si>
+  <si>
+    <t>Souleymane Diallo</t>
+  </si>
+  <si>
+    <t>Moustapha DIOUF</t>
+  </si>
+  <si>
+    <t>Tidiane Diallo</t>
+  </si>
+  <si>
+    <t>Ndiol NDIAYE</t>
+  </si>
+  <si>
+    <t>Grand Boutique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pour essayer </t>
+  </si>
+  <si>
+    <t>Médina</t>
+  </si>
+  <si>
+    <t>Diop et Frères</t>
+  </si>
+  <si>
+    <t>Café Altimo pot 100g x 24 pcs</t>
+  </si>
+  <si>
+    <t>Ouakam</t>
+  </si>
+  <si>
+    <t>Ibrahima Sori Diallo</t>
+  </si>
+  <si>
+    <t>Niang et frère</t>
+  </si>
+  <si>
+    <t>Bala</t>
+  </si>
+  <si>
+    <t>Moustapha Mbaye</t>
+  </si>
+  <si>
+    <t>Grand Yoff</t>
+  </si>
+  <si>
+    <t>Dame DIOP</t>
+  </si>
+  <si>
+    <t>Alune Ndiaye</t>
+  </si>
+  <si>
+    <t>Mouhamed KANTE</t>
+  </si>
+  <si>
+    <t>Zone de captage</t>
+  </si>
+  <si>
+    <t>Ousmane Dramé</t>
+  </si>
+  <si>
+    <t>Raa</t>
+  </si>
+  <si>
+    <t>Kolda</t>
+  </si>
+  <si>
+    <t>Mansour</t>
+  </si>
+  <si>
+    <t>Moustapha  seye</t>
+  </si>
+  <si>
+    <t>Mor seye</t>
+  </si>
+  <si>
+    <t>Mouhamed Diallo</t>
+  </si>
+  <si>
+    <t>Il veut essayer le produit mais il demande de revoir le prix il dit que c'est cher</t>
+  </si>
+  <si>
+    <t>KamLac Lait concentré sucré 24x1kg</t>
+  </si>
+  <si>
+    <t>Abdou Diop</t>
+  </si>
+  <si>
+    <t>Seye et Frère</t>
+  </si>
+  <si>
+    <t>Il dit que le produit est cher c'est pourquoi il ne peut pas prendre en grande quantité</t>
+  </si>
+  <si>
+    <t>Meadow Cup sac 25kg</t>
   </si>
 </sst>
 </file>
@@ -525,7 +660,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -546,11 +681,46 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -589,9 +759,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -599,6 +766,28 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -903,8 +1092,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}" name="Semaine_1" displayName="Semaine_1" ref="A1:P82" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16">
-  <autoFilter ref="A1:P82" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}" name="Semaine_1" displayName="Semaine_1" ref="A1:P124" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16">
+  <autoFilter ref="A1:P124" xr:uid="{FC757211-1341-459A-BE29-FAC5D7146FA5}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{F85C405C-E78B-4DA6-8568-08107D7551E4}" name="Date" dataDxfId="15"/>
     <tableColumn id="2" xr3:uid="{24A95AD6-D6B8-4864-9451-50BFB3565C62}" name="Prenom_Nom_RZ" dataDxfId="14"/>
@@ -1217,7 +1406,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Feuil2"/>
-  <dimension ref="A1:P82"/>
+  <dimension ref="A1:P124"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.53125" bestFit="1" customWidth="1"/>
@@ -4304,1189 +4493,3373 @@
       </c>
     </row>
     <row r="60" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A60" s="12">
+      <c r="A60" s="8">
         <v>46158</v>
       </c>
-      <c r="B60" s="13" t="s">
+      <c r="B60" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C60" s="13" t="s">
+      <c r="C60" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D60" s="13" t="s">
+      <c r="D60" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E60" s="13" t="s">
+      <c r="E60" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="F60" s="14">
+      <c r="F60" s="10">
         <v>781316258</v>
       </c>
-      <c r="G60" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H60" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I60" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J60" s="13" t="s">
+      <c r="G60" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H60" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I60" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J60" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="K60" s="13" t="s">
+      <c r="K60" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="L60" s="13">
+      <c r="L60" s="9">
         <v>60</v>
       </c>
-      <c r="M60" s="15">
+      <c r="M60" s="11">
         <v>9000</v>
       </c>
-      <c r="N60" s="15">
+      <c r="N60" s="11">
         <v>540000</v>
       </c>
-      <c r="O60" s="16" t="str">
+      <c r="O60" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P60" s="17" t="str">
+      <c r="P60" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="61" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A61" s="12">
+      <c r="A61" s="8">
         <v>46158</v>
       </c>
-      <c r="B61" s="13" t="s">
+      <c r="B61" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C61" s="13" t="s">
+      <c r="C61" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D61" s="13" t="s">
+      <c r="D61" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E61" s="13" t="s">
+      <c r="E61" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="F61" s="14">
+      <c r="F61" s="10">
         <v>781316258</v>
       </c>
-      <c r="G61" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H61" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I61" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J61" s="13" t="s">
+      <c r="G61" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H61" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I61" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J61" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="K61" s="13" t="s">
+      <c r="K61" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="L61" s="13">
+      <c r="L61" s="9">
         <v>10</v>
       </c>
-      <c r="M61" s="15">
+      <c r="M61" s="11">
         <v>9000</v>
       </c>
-      <c r="N61" s="15">
+      <c r="N61" s="11">
         <v>90000</v>
       </c>
-      <c r="O61" s="16" t="str">
+      <c r="O61" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P61" s="17" t="str">
+      <c r="P61" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="62" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A62" s="12">
+      <c r="A62" s="8">
         <v>46157</v>
       </c>
-      <c r="B62" s="13" t="s">
+      <c r="B62" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C62" s="13" t="s">
+      <c r="C62" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D62" s="13" t="s">
+      <c r="D62" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E62" s="13" t="s">
+      <c r="E62" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="F62" s="14">
+      <c r="F62" s="10">
         <v>776149093</v>
       </c>
-      <c r="G62" s="13" t="s">
+      <c r="G62" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H62" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I62" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J62" s="13" t="s">
+      <c r="H62" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I62" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J62" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="K62" s="13" t="s">
+      <c r="K62" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="L62" s="13">
+      <c r="L62" s="9">
         <v>25</v>
       </c>
-      <c r="M62" s="15">
+      <c r="M62" s="11">
         <v>6000</v>
       </c>
-      <c r="N62" s="15">
+      <c r="N62" s="11">
         <v>150000</v>
       </c>
-      <c r="O62" s="16" t="str">
+      <c r="O62" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P62" s="17" t="str">
+      <c r="P62" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="63" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A63" s="12">
+      <c r="A63" s="8">
         <v>46157</v>
       </c>
-      <c r="B63" s="13" t="s">
+      <c r="B63" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C63" s="13" t="s">
+      <c r="C63" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D63" s="13" t="s">
+      <c r="D63" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="E63" s="13" t="s">
+      <c r="E63" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="F63" s="14">
+      <c r="F63" s="10">
         <v>773012416</v>
       </c>
-      <c r="G63" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H63" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I63" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J63" s="13" t="s">
+      <c r="G63" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H63" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I63" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J63" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="K63" s="13" t="s">
+      <c r="K63" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="L63" s="13">
+      <c r="L63" s="9">
         <v>25</v>
       </c>
-      <c r="M63" s="15">
+      <c r="M63" s="11">
         <v>12000</v>
       </c>
-      <c r="N63" s="15">
+      <c r="N63" s="11">
         <v>300000</v>
       </c>
-      <c r="O63" s="16" t="str">
+      <c r="O63" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P63" s="17" t="str">
+      <c r="P63" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="64" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A64" s="12">
+      <c r="A64" s="8">
         <v>46157</v>
       </c>
-      <c r="B64" s="13" t="s">
+      <c r="B64" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C64" s="13" t="s">
+      <c r="C64" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D64" s="13" t="s">
+      <c r="D64" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="E64" s="13" t="s">
+      <c r="E64" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="F64" s="14">
+      <c r="F64" s="10">
         <v>773178746</v>
       </c>
-      <c r="G64" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H64" s="13" t="s">
+      <c r="G64" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H64" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="I64" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J64" s="13" t="s">
+      <c r="I64" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J64" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="K64" s="13" t="s">
+      <c r="K64" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="L64" s="13">
+      <c r="L64" s="9">
         <v>27</v>
       </c>
-      <c r="M64" s="15">
+      <c r="M64" s="11">
         <v>9000</v>
       </c>
-      <c r="N64" s="15">
+      <c r="N64" s="11">
         <v>243000</v>
       </c>
-      <c r="O64" s="16" t="str">
+      <c r="O64" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P64" s="17" t="str">
+      <c r="P64" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="65" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A65" s="12">
+      <c r="A65" s="8">
         <v>46157</v>
       </c>
-      <c r="B65" s="13" t="s">
+      <c r="B65" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C65" s="13" t="s">
+      <c r="C65" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D65" s="13" t="s">
+      <c r="D65" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="E65" s="13" t="s">
+      <c r="E65" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="F65" s="14">
+      <c r="F65" s="10">
         <v>773701528</v>
       </c>
-      <c r="G65" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H65" s="13" t="s">
+      <c r="G65" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H65" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="I65" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J65" s="13" t="s">
+      <c r="I65" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J65" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="K65" s="13" t="s">
+      <c r="K65" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="L65" s="13">
+      <c r="L65" s="9">
         <v>6</v>
       </c>
-      <c r="M65" s="15">
+      <c r="M65" s="11">
         <v>12000</v>
       </c>
-      <c r="N65" s="15">
+      <c r="N65" s="11">
         <v>72000</v>
       </c>
-      <c r="O65" s="16" t="str">
+      <c r="O65" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P65" s="17" t="str">
+      <c r="P65" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="66" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A66" s="12">
+      <c r="A66" s="8">
         <v>46157</v>
       </c>
-      <c r="B66" s="13" t="s">
+      <c r="B66" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C66" s="13" t="s">
+      <c r="C66" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D66" s="13" t="s">
+      <c r="D66" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="E66" s="13" t="s">
+      <c r="E66" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="F66" s="14">
+      <c r="F66" s="10">
         <v>765956010</v>
       </c>
-      <c r="G66" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H66" s="13" t="s">
+      <c r="G66" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H66" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="I66" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J66" s="13" t="s">
+      <c r="I66" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J66" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="K66" s="13" t="s">
+      <c r="K66" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="L66" s="13">
+      <c r="L66" s="9">
         <v>10</v>
       </c>
-      <c r="M66" s="15">
+      <c r="M66" s="11">
         <v>9000</v>
       </c>
-      <c r="N66" s="15">
+      <c r="N66" s="11">
         <v>90000</v>
       </c>
-      <c r="O66" s="16" t="str">
+      <c r="O66" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P66" s="17" t="str">
+      <c r="P66" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="67" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A67" s="12">
+      <c r="A67" s="8">
         <v>46156</v>
       </c>
-      <c r="B67" s="13" t="s">
+      <c r="B67" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C67" s="13" t="s">
+      <c r="C67" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D67" s="13" t="s">
+      <c r="D67" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E67" s="13" t="s">
+      <c r="E67" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="F67" s="14">
+      <c r="F67" s="10">
         <v>781282357</v>
       </c>
-      <c r="G67" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H67" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I67" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J67" s="13" t="s">
+      <c r="G67" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H67" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I67" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J67" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="K67" s="13" t="s">
+      <c r="K67" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="L67" s="13">
+      <c r="L67" s="9">
         <v>50</v>
       </c>
-      <c r="M67" s="15">
+      <c r="M67" s="11">
         <v>26000</v>
       </c>
-      <c r="N67" s="15">
+      <c r="N67" s="11">
         <v>1300000</v>
       </c>
-      <c r="O67" s="16" t="str">
+      <c r="O67" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P67" s="17" t="str">
+      <c r="P67" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="68" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A68" s="12">
+      <c r="A68" s="8">
         <v>46156</v>
       </c>
-      <c r="B68" s="13" t="s">
+      <c r="B68" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C68" s="13" t="s">
+      <c r="C68" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D68" s="13" t="s">
+      <c r="D68" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E68" s="13" t="s">
+      <c r="E68" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="F68" s="14">
+      <c r="F68" s="10">
         <v>762974040</v>
       </c>
-      <c r="G68" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H68" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I68" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J68" s="13" t="s">
+      <c r="G68" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H68" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I68" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J68" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="K68" s="13" t="s">
+      <c r="K68" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="L68" s="13">
+      <c r="L68" s="9">
         <v>25</v>
       </c>
-      <c r="M68" s="15">
+      <c r="M68" s="11">
         <v>26000</v>
       </c>
-      <c r="N68" s="15">
+      <c r="N68" s="11">
         <v>650000</v>
       </c>
-      <c r="O68" s="16" t="str">
+      <c r="O68" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P68" s="17" t="str">
+      <c r="P68" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="69" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A69" s="12">
+      <c r="A69" s="8">
         <v>46156</v>
       </c>
-      <c r="B69" s="13" t="s">
+      <c r="B69" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C69" s="13" t="s">
+      <c r="C69" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D69" s="13" t="s">
+      <c r="D69" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E69" s="13" t="s">
+      <c r="E69" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="F69" s="14">
+      <c r="F69" s="10">
         <v>775411094</v>
       </c>
-      <c r="G69" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H69" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I69" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J69" s="13" t="s">
+      <c r="G69" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H69" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I69" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J69" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="K69" s="13" t="s">
+      <c r="K69" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="L69" s="13">
+      <c r="L69" s="9">
         <v>100</v>
       </c>
-      <c r="M69" s="15">
+      <c r="M69" s="11">
         <v>9000</v>
       </c>
-      <c r="N69" s="15">
+      <c r="N69" s="11">
         <v>900000</v>
       </c>
-      <c r="O69" s="16" t="str">
+      <c r="O69" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P69" s="17" t="str">
+      <c r="P69" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="70" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A70" s="12">
+      <c r="A70" s="8">
         <v>46156</v>
       </c>
-      <c r="B70" s="13" t="s">
+      <c r="B70" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C70" s="13" t="s">
+      <c r="C70" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D70" s="13" t="s">
+      <c r="D70" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E70" s="13" t="s">
+      <c r="E70" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="F70" s="14">
+      <c r="F70" s="10">
         <v>775264622</v>
       </c>
-      <c r="G70" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H70" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I70" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J70" s="13" t="s">
+      <c r="G70" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H70" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I70" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J70" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="K70" s="13" t="s">
+      <c r="K70" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="L70" s="13">
+      <c r="L70" s="9">
         <v>25</v>
       </c>
-      <c r="M70" s="15">
+      <c r="M70" s="11">
         <v>26000</v>
       </c>
-      <c r="N70" s="15">
+      <c r="N70" s="11">
         <v>650000</v>
       </c>
-      <c r="O70" s="16" t="str">
+      <c r="O70" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P70" s="17" t="str">
+      <c r="P70" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A71" s="12">
+      <c r="A71" s="8">
         <v>46155</v>
       </c>
-      <c r="B71" s="13" t="s">
+      <c r="B71" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C71" s="13" t="s">
+      <c r="C71" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D71" s="13" t="s">
+      <c r="D71" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="E71" s="13" t="s">
+      <c r="E71" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="F71" s="14">
+      <c r="F71" s="10">
         <v>775987400</v>
       </c>
-      <c r="G71" s="13" t="s">
+      <c r="G71" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H71" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I71" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J71" s="13" t="s">
+      <c r="H71" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I71" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J71" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="K71" s="13" t="s">
+      <c r="K71" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="L71" s="13">
+      <c r="L71" s="9">
         <v>2</v>
       </c>
-      <c r="M71" s="15">
+      <c r="M71" s="11">
         <v>9000</v>
       </c>
-      <c r="N71" s="15">
+      <c r="N71" s="11">
         <v>18000</v>
       </c>
-      <c r="O71" s="16" t="str">
+      <c r="O71" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P71" s="17" t="str">
+      <c r="P71" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A72" s="12">
+      <c r="A72" s="8">
         <v>46155</v>
       </c>
-      <c r="B72" s="13" t="s">
+      <c r="B72" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C72" s="13" t="s">
+      <c r="C72" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D72" s="13" t="s">
+      <c r="D72" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="E72" s="13" t="s">
+      <c r="E72" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="F72" s="14">
+      <c r="F72" s="10">
         <v>775987400</v>
       </c>
-      <c r="G72" s="13" t="s">
+      <c r="G72" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H72" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I72" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J72" s="13" t="s">
+      <c r="H72" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I72" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J72" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="K72" s="13" t="s">
+      <c r="K72" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L72" s="13">
+      <c r="L72" s="9">
         <v>4</v>
       </c>
-      <c r="M72" s="15">
+      <c r="M72" s="11">
         <v>19500</v>
       </c>
-      <c r="N72" s="15">
+      <c r="N72" s="11">
         <v>78000</v>
       </c>
-      <c r="O72" s="16" t="str">
+      <c r="O72" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P72" s="17" t="str">
+      <c r="P72" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="73" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A73" s="12">
+      <c r="A73" s="8">
         <v>46155</v>
       </c>
-      <c r="B73" s="13" t="s">
+      <c r="B73" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C73" s="13" t="s">
+      <c r="C73" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D73" s="13" t="s">
+      <c r="D73" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="E73" s="13" t="s">
+      <c r="E73" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="F73" s="14">
+      <c r="F73" s="10">
         <v>775426848</v>
       </c>
-      <c r="G73" s="13" t="s">
+      <c r="G73" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H73" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I73" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J73" s="13" t="s">
+      <c r="H73" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I73" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J73" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="K73" s="13" t="s">
+      <c r="K73" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L73" s="13">
+      <c r="L73" s="9">
         <v>8</v>
       </c>
-      <c r="M73" s="15">
+      <c r="M73" s="11">
         <v>19500</v>
       </c>
-      <c r="N73" s="15">
+      <c r="N73" s="11">
         <v>156000</v>
       </c>
-      <c r="O73" s="16" t="str">
+      <c r="O73" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P73" s="17" t="str">
+      <c r="P73" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A74" s="12">
+      <c r="A74" s="8">
         <v>46155</v>
       </c>
-      <c r="B74" s="13" t="s">
+      <c r="B74" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C74" s="13" t="s">
+      <c r="C74" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="D74" s="13" t="s">
+      <c r="D74" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E74" s="13" t="s">
+      <c r="E74" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="F74" s="14">
+      <c r="F74" s="10">
         <v>770712599</v>
       </c>
-      <c r="G74" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H74" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I74" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J74" s="13" t="s">
+      <c r="G74" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H74" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I74" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J74" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="K74" s="13" t="s">
+      <c r="K74" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="L74" s="13">
+      <c r="L74" s="9">
         <v>100</v>
       </c>
-      <c r="M74" s="15">
+      <c r="M74" s="11">
         <v>26000</v>
       </c>
-      <c r="N74" s="15">
+      <c r="N74" s="11">
         <v>2600000</v>
       </c>
-      <c r="O74" s="16" t="str">
+      <c r="O74" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P74" s="17" t="str">
+      <c r="P74" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A75" s="12">
+      <c r="A75" s="8">
         <v>46154</v>
       </c>
-      <c r="B75" s="13" t="s">
+      <c r="B75" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C75" s="13" t="s">
+      <c r="C75" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D75" s="13" t="s">
+      <c r="D75" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E75" s="13" t="s">
+      <c r="E75" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F75" s="14">
+      <c r="F75" s="10">
         <v>776634479</v>
       </c>
-      <c r="G75" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H75" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I75" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J75" s="13" t="s">
+      <c r="G75" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H75" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I75" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J75" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="K75" s="13" t="s">
+      <c r="K75" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L75" s="13">
+      <c r="L75" s="9">
         <v>3</v>
       </c>
-      <c r="M75" s="15">
+      <c r="M75" s="11">
         <v>19500</v>
       </c>
-      <c r="N75" s="15">
+      <c r="N75" s="11">
         <v>58500</v>
       </c>
-      <c r="O75" s="16" t="str">
+      <c r="O75" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P75" s="17" t="str">
+      <c r="P75" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="76" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A76" s="12">
+      <c r="A76" s="8">
         <v>46154</v>
       </c>
-      <c r="B76" s="13" t="s">
+      <c r="B76" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C76" s="13" t="s">
+      <c r="C76" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D76" s="13" t="s">
+      <c r="D76" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="E76" s="13" t="s">
+      <c r="E76" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="F76" s="14">
+      <c r="F76" s="10">
         <v>778195274</v>
       </c>
-      <c r="G76" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H76" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I76" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J76" s="13" t="s">
+      <c r="G76" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H76" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I76" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J76" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="K76" s="13" t="s">
+      <c r="K76" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="L76" s="13">
+      <c r="L76" s="9">
         <v>100</v>
       </c>
-      <c r="M76" s="15">
+      <c r="M76" s="11">
         <v>26000</v>
       </c>
-      <c r="N76" s="15">
+      <c r="N76" s="11">
         <v>2600000</v>
       </c>
-      <c r="O76" s="16" t="str">
+      <c r="O76" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P76" s="17" t="str">
+      <c r="P76" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.45">
-      <c r="A77" s="12">
+      <c r="A77" s="8">
         <v>46154</v>
       </c>
-      <c r="B77" s="13" t="s">
+      <c r="B77" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C77" s="13" t="s">
+      <c r="C77" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D77" s="13" t="s">
+      <c r="D77" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E77" s="13" t="s">
+      <c r="E77" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="F77" s="14">
+      <c r="F77" s="10">
         <v>773564759</v>
       </c>
-      <c r="G77" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H77" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I77" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J77" s="13" t="s">
+      <c r="G77" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H77" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I77" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J77" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="K77" s="13" t="s">
+      <c r="K77" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="L77" s="13">
+      <c r="L77" s="9">
         <v>10</v>
       </c>
-      <c r="M77" s="15">
+      <c r="M77" s="11">
         <v>19500</v>
       </c>
-      <c r="N77" s="15">
+      <c r="N77" s="11">
         <v>195000</v>
       </c>
-      <c r="O77" s="16" t="str">
+      <c r="O77" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P77" s="17" t="str">
+      <c r="P77" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="78" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A78" s="12">
+      <c r="A78" s="8">
         <v>46154</v>
       </c>
-      <c r="B78" s="13" t="s">
+      <c r="B78" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C78" s="13" t="s">
+      <c r="C78" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D78" s="13" t="s">
+      <c r="D78" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E78" s="13" t="s">
+      <c r="E78" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F78" s="14">
+      <c r="F78" s="10">
         <v>776634479</v>
       </c>
-      <c r="G78" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H78" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I78" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J78" s="13" t="s">
+      <c r="G78" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H78" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I78" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J78" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="K78" s="13" t="s">
+      <c r="K78" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="L78" s="13">
+      <c r="L78" s="9">
         <v>1</v>
       </c>
-      <c r="M78" s="15">
+      <c r="M78" s="11">
         <v>15000</v>
       </c>
-      <c r="N78" s="15">
+      <c r="N78" s="11">
         <v>15000</v>
       </c>
-      <c r="O78" s="16" t="str">
+      <c r="O78" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P78" s="17" t="str">
+      <c r="P78" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="79" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A79" s="12">
+      <c r="A79" s="8">
         <v>46153</v>
       </c>
-      <c r="B79" s="13" t="s">
+      <c r="B79" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C79" s="13" t="s">
+      <c r="C79" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D79" s="13" t="s">
+      <c r="D79" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="E79" s="13" t="s">
+      <c r="E79" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="F79" s="14">
+      <c r="F79" s="10">
         <v>785459209</v>
       </c>
-      <c r="G79" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H79" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I79" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J79" s="13" t="s">
+      <c r="G79" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H79" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I79" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J79" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="K79" s="13" t="s">
+      <c r="K79" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="L79" s="13">
+      <c r="L79" s="9">
         <v>25</v>
       </c>
-      <c r="M79" s="15">
+      <c r="M79" s="11">
         <v>26000</v>
       </c>
-      <c r="N79" s="15">
+      <c r="N79" s="11">
         <v>650000</v>
       </c>
-      <c r="O79" s="16" t="str">
+      <c r="O79" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P79" s="17" t="str">
+      <c r="P79" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="80" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A80" s="12">
+      <c r="A80" s="8">
         <v>46153</v>
       </c>
-      <c r="B80" s="13" t="s">
+      <c r="B80" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C80" s="13" t="s">
+      <c r="C80" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D80" s="13" t="s">
+      <c r="D80" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E80" s="13" t="s">
+      <c r="E80" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F80" s="14">
+      <c r="F80" s="10">
         <v>776428218</v>
       </c>
-      <c r="G80" s="13" t="s">
+      <c r="G80" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H80" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I80" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J80" s="13" t="s">
+      <c r="H80" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I80" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J80" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="K80" s="13" t="s">
+      <c r="K80" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="L80" s="13">
+      <c r="L80" s="9">
         <v>778</v>
       </c>
-      <c r="M80" s="15">
+      <c r="M80" s="11">
         <v>7500</v>
       </c>
-      <c r="N80" s="15">
+      <c r="N80" s="11">
         <v>5835000</v>
       </c>
-      <c r="O80" s="16" t="str">
+      <c r="O80" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P80" s="17" t="str">
+      <c r="P80" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="81" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A81" s="12">
+      <c r="A81" s="8">
         <v>46153</v>
       </c>
-      <c r="B81" s="13" t="s">
+      <c r="B81" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C81" s="13" t="s">
+      <c r="C81" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D81" s="13" t="s">
+      <c r="D81" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E81" s="13" t="s">
+      <c r="E81" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F81" s="14">
+      <c r="F81" s="10">
         <v>776428218</v>
       </c>
-      <c r="G81" s="13" t="s">
+      <c r="G81" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H81" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I81" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J81" s="13" t="s">
+      <c r="H81" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I81" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J81" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="K81" s="13" t="s">
+      <c r="K81" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="L81" s="13">
+      <c r="L81" s="9">
         <v>25</v>
       </c>
-      <c r="M81" s="15">
+      <c r="M81" s="11">
         <v>8750</v>
       </c>
-      <c r="N81" s="15">
+      <c r="N81" s="11">
         <v>218750</v>
       </c>
-      <c r="O81" s="16" t="str">
+      <c r="O81" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P81" s="17" t="str">
+      <c r="P81" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>
     </row>
     <row r="82" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
-      <c r="A82" s="12">
+      <c r="A82" s="8">
         <v>46158</v>
       </c>
-      <c r="B82" s="13" t="s">
+      <c r="B82" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C82" s="13" t="s">
+      <c r="C82" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D82" s="13" t="s">
+      <c r="D82" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E82" s="13" t="s">
+      <c r="E82" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="F82" s="14">
+      <c r="F82" s="10">
         <v>778657940</v>
       </c>
-      <c r="G82" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="H82" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I82" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J82" s="13" t="s">
+      <c r="G82" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H82" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I82" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="J82" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="K82" s="13"/>
-      <c r="L82" s="13"/>
-      <c r="M82" s="15"/>
-      <c r="N82" s="15"/>
-      <c r="O82" s="16" t="str">
+      <c r="K82" s="9"/>
+      <c r="L82" s="9"/>
+      <c r="M82" s="11"/>
+      <c r="N82" s="11"/>
+      <c r="O82" s="7" t="str">
         <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
         <v>S20</v>
       </c>
-      <c r="P82" s="17" t="str">
+      <c r="P82" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A83" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B83" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C83" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D83" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="E83" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="F83" s="13">
+        <v>779235028</v>
+      </c>
+      <c r="G83" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H83" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I83" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J83" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="K83" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L83" s="13">
+        <v>33</v>
+      </c>
+      <c r="M83" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N83" s="14">
+        <v>858000</v>
+      </c>
+      <c r="O83" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P83" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A84" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B84" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C84" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D84" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E84" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="F84" s="13">
+        <v>770217868</v>
+      </c>
+      <c r="G84" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H84" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I84" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J84" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="K84" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L84" s="13">
+        <v>25</v>
+      </c>
+      <c r="M84" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N84" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O84" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P84" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A85" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B85" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C85" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D85" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E85" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="F85" s="13">
+        <v>774289051</v>
+      </c>
+      <c r="G85" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H85" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I85" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J85" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="K85" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L85" s="13">
+        <v>25</v>
+      </c>
+      <c r="M85" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N85" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O85" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P85" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A86" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B86" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C86" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D86" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="E86" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="F86" s="13">
+        <v>771701320</v>
+      </c>
+      <c r="G86" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H86" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I86" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J86" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="K86" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="L86" s="13">
+        <v>25</v>
+      </c>
+      <c r="M86" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N86" s="14">
+        <v>225000</v>
+      </c>
+      <c r="O86" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P86" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A87" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B87" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C87" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D87" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="E87" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="F87" s="13">
+        <v>771701320</v>
+      </c>
+      <c r="G87" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H87" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I87" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J87" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="K87" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L87" s="13">
+        <v>25</v>
+      </c>
+      <c r="M87" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N87" s="14">
+        <v>225000</v>
+      </c>
+      <c r="O87" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P87" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A88" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B88" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C88" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D88" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E88" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="F88" s="13">
+        <v>771619220</v>
+      </c>
+      <c r="G88" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H88" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I88" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J88" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="K88" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L88" s="13">
+        <v>51</v>
+      </c>
+      <c r="M88" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N88" s="14">
+        <v>1326000</v>
+      </c>
+      <c r="O88" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P88" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A89" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B89" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C89" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D89" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="E89" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="F89" s="13">
+        <v>784785900</v>
+      </c>
+      <c r="G89" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H89" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I89" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J89" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="K89" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L89" s="13">
+        <v>100</v>
+      </c>
+      <c r="M89" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N89" s="14">
+        <v>2600000</v>
+      </c>
+      <c r="O89" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P89" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="90" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A90" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B90" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C90" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D90" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="E90" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="F90" s="13">
+        <v>779110400</v>
+      </c>
+      <c r="G90" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H90" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I90" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J90" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="K90" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L90" s="13">
+        <v>34</v>
+      </c>
+      <c r="M90" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N90" s="14">
+        <v>884000</v>
+      </c>
+      <c r="O90" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P90" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="91" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A91" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B91" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C91" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D91" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="E91" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="F91" s="13">
+        <v>763357265</v>
+      </c>
+      <c r="G91" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H91" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I91" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J91" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="K91" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L91" s="13">
+        <v>1</v>
+      </c>
+      <c r="M91" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N91" s="14">
+        <v>26000</v>
+      </c>
+      <c r="O91" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P91" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="92" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A92" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B92" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C92" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D92" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="E92" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="F92" s="13">
+        <v>771155837</v>
+      </c>
+      <c r="G92" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H92" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I92" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J92" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="K92" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L92" s="13">
+        <v>3</v>
+      </c>
+      <c r="M92" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N92" s="14">
+        <v>78000</v>
+      </c>
+      <c r="O92" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P92" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="93" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A93" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B93" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C93" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D93" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="E93" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="F93" s="13">
+        <v>763030898</v>
+      </c>
+      <c r="G93" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H93" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I93" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J93" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="K93" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L93" s="13">
+        <v>2</v>
+      </c>
+      <c r="M93" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N93" s="14">
+        <v>52000</v>
+      </c>
+      <c r="O93" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P93" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="94" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A94" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B94" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C94" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D94" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="E94" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="F94" s="13">
+        <v>785852626</v>
+      </c>
+      <c r="G94" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H94" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I94" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J94" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="K94" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L94" s="13">
+        <v>33</v>
+      </c>
+      <c r="M94" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N94" s="14">
+        <v>858000</v>
+      </c>
+      <c r="O94" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P94" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="95" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A95" s="12">
+        <v>46161</v>
+      </c>
+      <c r="B95" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C95" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D95" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="E95" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F95" s="13">
+        <v>776874747</v>
+      </c>
+      <c r="G95" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H95" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I95" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J95" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="K95" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L95" s="13">
+        <v>25</v>
+      </c>
+      <c r="M95" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N95" s="14">
+        <v>225000</v>
+      </c>
+      <c r="O95" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P95" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="96" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A96" s="12">
+        <v>46161</v>
+      </c>
+      <c r="B96" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C96" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D96" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="E96" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="F96" s="13">
+        <v>764883712</v>
+      </c>
+      <c r="G96" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="H96" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I96" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J96" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="K96" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L96" s="13">
+        <v>5</v>
+      </c>
+      <c r="M96" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N96" s="14">
+        <v>45000</v>
+      </c>
+      <c r="O96" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P96" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="97" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A97" s="12">
+        <v>46161</v>
+      </c>
+      <c r="B97" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C97" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D97" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="E97" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="F97" s="13">
+        <v>776347177</v>
+      </c>
+      <c r="G97" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H97" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I97" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J97" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="K97" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L97" s="13">
+        <v>5</v>
+      </c>
+      <c r="M97" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N97" s="14">
+        <v>130000</v>
+      </c>
+      <c r="O97" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P97" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="98" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A98" s="12">
+        <v>46161</v>
+      </c>
+      <c r="B98" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C98" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D98" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="E98" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="F98" s="13">
+        <v>776347177</v>
+      </c>
+      <c r="G98" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H98" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I98" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J98" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="K98" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="L98" s="13">
+        <v>1</v>
+      </c>
+      <c r="M98" s="14">
+        <v>33500</v>
+      </c>
+      <c r="N98" s="14">
+        <v>33500</v>
+      </c>
+      <c r="O98" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P98" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="99" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A99" s="12">
+        <v>46161</v>
+      </c>
+      <c r="B99" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C99" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D99" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="E99" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="F99" s="13">
+        <v>775623289</v>
+      </c>
+      <c r="G99" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H99" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I99" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J99" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="K99" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L99" s="13">
+        <v>20</v>
+      </c>
+      <c r="M99" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N99" s="14">
+        <v>520000</v>
+      </c>
+      <c r="O99" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P99" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="100" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A100" s="12">
+        <v>46161</v>
+      </c>
+      <c r="B100" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C100" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D100" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="E100" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="F100" s="13">
+        <v>775623289</v>
+      </c>
+      <c r="G100" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H100" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I100" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J100" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="K100" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L100" s="13">
+        <v>25</v>
+      </c>
+      <c r="M100" s="14">
+        <v>19500</v>
+      </c>
+      <c r="N100" s="14">
+        <v>487500</v>
+      </c>
+      <c r="O100" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P100" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="101" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A101" s="12">
+        <v>46160</v>
+      </c>
+      <c r="B101" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C101" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D101" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E101" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="F101" s="13">
+        <v>776536527</v>
+      </c>
+      <c r="G101" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H101" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I101" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J101" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="K101" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="L101" s="13">
+        <v>15</v>
+      </c>
+      <c r="M101" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N101" s="14">
+        <v>135000</v>
+      </c>
+      <c r="O101" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P101" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="102" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A102" s="12">
+        <v>46160</v>
+      </c>
+      <c r="B102" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C102" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D102" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="E102" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="F102" s="13">
+        <v>776175166</v>
+      </c>
+      <c r="G102" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H102" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I102" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J102" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="K102" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L102" s="13">
+        <v>100</v>
+      </c>
+      <c r="M102" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N102" s="14">
+        <v>2600000</v>
+      </c>
+      <c r="O102" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P102" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="103" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A103" s="12">
+        <v>46160</v>
+      </c>
+      <c r="B103" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C103" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D103" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E103" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="F103" s="13">
+        <v>776536527</v>
+      </c>
+      <c r="G103" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H103" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I103" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J103" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="K103" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L103" s="13">
+        <v>15</v>
+      </c>
+      <c r="M103" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N103" s="14">
+        <v>135000</v>
+      </c>
+      <c r="O103" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P103" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="104" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A104" s="12">
+        <v>46160</v>
+      </c>
+      <c r="B104" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C104" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D104" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E104" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="F104" s="13">
+        <v>772899294</v>
+      </c>
+      <c r="G104" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H104" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I104" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J104" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="K104" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L104" s="13">
+        <v>25</v>
+      </c>
+      <c r="M104" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N104" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O104" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P104" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="105" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A105" s="17">
+        <v>46161</v>
+      </c>
+      <c r="B105" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C105" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="D105" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="E105" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="F105" s="19">
+        <v>774216339</v>
+      </c>
+      <c r="G105" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H105" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="I105" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="J105" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="K105" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="L105" s="18">
+        <v>25</v>
+      </c>
+      <c r="M105" s="20">
+        <v>26000</v>
+      </c>
+      <c r="N105" s="21">
+        <v>650000</v>
+      </c>
+      <c r="O105" s="22" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P105" s="23" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="106" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A106" s="12">
+        <v>46162</v>
+      </c>
+      <c r="B106" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C106" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D106" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E106" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="F106" s="24">
+        <v>775273147</v>
+      </c>
+      <c r="G106" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H106" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I106" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J106" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="K106" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="L106" s="13">
+        <v>100</v>
+      </c>
+      <c r="M106" s="14">
+        <v>5750</v>
+      </c>
+      <c r="N106" s="14">
+        <v>575000</v>
+      </c>
+      <c r="O106" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P106" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="107" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A107" s="12">
+        <v>46165</v>
+      </c>
+      <c r="B107" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C107" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D107" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E107" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="F107" s="24">
+        <v>777096402</v>
+      </c>
+      <c r="G107" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H107" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I107" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J107" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="K107" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L107" s="13">
+        <v>50</v>
+      </c>
+      <c r="M107" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N107" s="14">
+        <v>450000</v>
+      </c>
+      <c r="O107" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P107" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="108" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A108" s="12">
+        <v>46165</v>
+      </c>
+      <c r="B108" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C108" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D108" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="E108" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="F108" s="24">
+        <v>775544532</v>
+      </c>
+      <c r="G108" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H108" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I108" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J108" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="K108" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L108" s="13">
+        <v>25</v>
+      </c>
+      <c r="M108" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N108" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O108" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P108" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="109" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A109" s="12">
+        <v>46165</v>
+      </c>
+      <c r="B109" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C109" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D109" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="E109" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="F109" s="24">
+        <v>773739328</v>
+      </c>
+      <c r="G109" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H109" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I109" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J109" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="K109" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L109" s="13">
+        <v>10</v>
+      </c>
+      <c r="M109" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N109" s="14">
+        <v>90000</v>
+      </c>
+      <c r="O109" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P109" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="110" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A110" s="12">
+        <v>46164</v>
+      </c>
+      <c r="B110" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C110" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D110" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="E110" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="F110" s="24">
+        <v>779414699</v>
+      </c>
+      <c r="G110" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H110" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I110" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J110" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="K110" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L110" s="13">
+        <v>15</v>
+      </c>
+      <c r="M110" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N110" s="14">
+        <v>135000</v>
+      </c>
+      <c r="O110" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P110" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="111" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A111" s="12">
+        <v>46164</v>
+      </c>
+      <c r="B111" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C111" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D111" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="E111" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="F111" s="24">
+        <v>779414699</v>
+      </c>
+      <c r="G111" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H111" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I111" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J111" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="K111" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="L111" s="13">
+        <v>10</v>
+      </c>
+      <c r="M111" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N111" s="14">
+        <v>90000</v>
+      </c>
+      <c r="O111" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P111" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="112" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A112" s="12">
+        <v>46164</v>
+      </c>
+      <c r="B112" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C112" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D112" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="E112" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="F112" s="24">
+        <v>772252177</v>
+      </c>
+      <c r="G112" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H112" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I112" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J112" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="K112" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L112" s="13">
+        <v>50</v>
+      </c>
+      <c r="M112" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N112" s="14">
+        <v>1300000</v>
+      </c>
+      <c r="O112" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P112" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="113" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A113" s="12">
+        <v>46164</v>
+      </c>
+      <c r="B113" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C113" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D113" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="E113" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="F113" s="24">
+        <v>775284696</v>
+      </c>
+      <c r="G113" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H113" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I113" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J113" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="K113" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L113" s="13">
+        <v>50</v>
+      </c>
+      <c r="M113" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N113" s="14">
+        <v>1300000</v>
+      </c>
+      <c r="O113" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P113" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="114" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A114" s="12">
+        <v>46164</v>
+      </c>
+      <c r="B114" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C114" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D114" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="E114" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="F114" s="24">
+        <v>765956010</v>
+      </c>
+      <c r="G114" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H114" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I114" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J114" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="K114" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="L114" s="13">
+        <v>5</v>
+      </c>
+      <c r="M114" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N114" s="14">
+        <v>45000</v>
+      </c>
+      <c r="O114" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P114" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="115" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A115" s="12">
+        <v>46164</v>
+      </c>
+      <c r="B115" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C115" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D115" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="E115" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="F115" s="24">
+        <v>765956010</v>
+      </c>
+      <c r="G115" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H115" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I115" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J115" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="K115" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L115" s="13">
+        <v>20</v>
+      </c>
+      <c r="M115" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N115" s="14">
+        <v>180000</v>
+      </c>
+      <c r="O115" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P115" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="116" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A116" s="12">
+        <v>46164</v>
+      </c>
+      <c r="B116" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C116" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D116" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E116" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="F116" s="24">
+        <v>775630094</v>
+      </c>
+      <c r="G116" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H116" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I116" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J116" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="K116" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="L116" s="13">
+        <v>25</v>
+      </c>
+      <c r="M116" s="14">
+        <v>28000</v>
+      </c>
+      <c r="N116" s="14">
+        <v>700000</v>
+      </c>
+      <c r="O116" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P116" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="117" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A117" s="12">
+        <v>46164</v>
+      </c>
+      <c r="B117" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C117" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D117" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E117" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="F117" s="24">
+        <v>774483791</v>
+      </c>
+      <c r="G117" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H117" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I117" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J117" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="K117" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="L117" s="13">
+        <v>5</v>
+      </c>
+      <c r="M117" s="14">
+        <v>28000</v>
+      </c>
+      <c r="N117" s="14">
+        <v>140000</v>
+      </c>
+      <c r="O117" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P117" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="118" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A118" s="12">
+        <v>46164</v>
+      </c>
+      <c r="B118" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C118" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D118" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E118" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="F118" s="24">
+        <v>777096402</v>
+      </c>
+      <c r="G118" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H118" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I118" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J118" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="K118" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L118" s="13">
+        <v>25</v>
+      </c>
+      <c r="M118" s="14">
+        <v>19500</v>
+      </c>
+      <c r="N118" s="14">
+        <v>487500</v>
+      </c>
+      <c r="O118" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P118" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="119" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A119" s="12">
+        <v>46163</v>
+      </c>
+      <c r="B119" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C119" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D119" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="E119" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="F119" s="24">
+        <v>783740441</v>
+      </c>
+      <c r="G119" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H119" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I119" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J119" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="K119" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="L119" s="13">
+        <v>10</v>
+      </c>
+      <c r="M119" s="14">
+        <v>9000</v>
+      </c>
+      <c r="N119" s="14">
+        <v>90000</v>
+      </c>
+      <c r="O119" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P119" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="120" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A120" s="12">
+        <v>46163</v>
+      </c>
+      <c r="B120" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C120" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D120" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E120" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="F120" s="24">
+        <v>770712599</v>
+      </c>
+      <c r="G120" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H120" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I120" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J120" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="K120" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="L120" s="13">
+        <v>100</v>
+      </c>
+      <c r="M120" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N120" s="14">
+        <v>2600000</v>
+      </c>
+      <c r="O120" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P120" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="121" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A121" s="12">
+        <v>46163</v>
+      </c>
+      <c r="B121" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C121" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D121" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="E121" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="F121" s="24">
+        <v>774216341</v>
+      </c>
+      <c r="G121" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H121" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I121" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J121" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="K121" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L121" s="13">
+        <v>5</v>
+      </c>
+      <c r="M121" s="14">
+        <v>19500</v>
+      </c>
+      <c r="N121" s="14">
+        <v>97500</v>
+      </c>
+      <c r="O121" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P121" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="122" spans="1:16" ht="28.15" x14ac:dyDescent="0.45">
+      <c r="A122" s="12">
+        <v>46163</v>
+      </c>
+      <c r="B122" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C122" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D122" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E122" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="F122" s="24">
+        <v>775485563</v>
+      </c>
+      <c r="G122" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H122" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I122" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J122" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="K122" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L122" s="13">
+        <v>10</v>
+      </c>
+      <c r="M122" s="14">
+        <v>19500</v>
+      </c>
+      <c r="N122" s="14">
+        <v>195000</v>
+      </c>
+      <c r="O122" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P122" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="123" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A123" s="12">
+        <v>46163</v>
+      </c>
+      <c r="B123" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C123" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D123" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="E123" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="F123" s="24">
+        <v>775544532</v>
+      </c>
+      <c r="G123" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H123" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I123" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J123" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="K123" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="L123" s="13">
+        <v>25</v>
+      </c>
+      <c r="M123" s="14">
+        <v>26000</v>
+      </c>
+      <c r="N123" s="14">
+        <v>650000</v>
+      </c>
+      <c r="O123" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P123" s="16" t="str">
+        <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
+        <v>mai</v>
+      </c>
+    </row>
+    <row r="124" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A124" s="12">
+        <v>46163</v>
+      </c>
+      <c r="B124" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C124" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D124" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="E124" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="F124" s="24">
+        <v>776634479</v>
+      </c>
+      <c r="G124" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="H124" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I124" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="J124" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="K124" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="L124" s="13">
+        <v>8</v>
+      </c>
+      <c r="M124" s="14">
+        <v>55000</v>
+      </c>
+      <c r="N124" s="14">
+        <v>440000</v>
+      </c>
+      <c r="O124" s="15" t="str">
+        <f>"S"&amp;_xlfn.ISOWEEKNUM(Semaine_1[[#This Row],[Date]])</f>
+        <v>S21</v>
+      </c>
+      <c r="P124" s="16" t="str">
         <f>TEXT(Semaine_1[[#This Row],[Date]],"MMMM")</f>
         <v>mai</v>
       </c>

</xml_diff>